<commit_message>
docs: updated the journal
</commit_message>
<xml_diff>
--- a/Annexes/Journal_de_travail/Journal_de_Travail_Léonard_Weber.xlsx
+++ b/Annexes/Journal_de_travail/Journal_de_Travail_Léonard_Weber.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduvaud-my.sharepoint.com/personal/pe04cuw_eduvaud_ch/Documents/CPNV_2025-2026/Semaine.projet.lego/journal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="292" documentId="13_ncr:1_{EFDCB34D-4D99-487E-82C9-6E7A8D14F32E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B1C19E3-5890-462F-B184-1A3C202D8E3B}"/>
+  <xr:revisionPtr revIDLastSave="362" documentId="13_ncr:1_{EFDCB34D-4D99-487E-82C9-6E7A8D14F32E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD85DE2C-997A-49C3-A803-5A211CE6396E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="160">
   <si>
     <t>Jour</t>
   </si>
@@ -86,9 +86,6 @@
     <t>Réalisation de la planification initiale</t>
   </si>
   <si>
-    <t>Réalisation des scénarios de type "guest"</t>
-  </si>
-  <si>
     <t>Retouches de la documentation</t>
   </si>
   <si>
@@ -500,7 +497,28 @@
     <t>natan m'a aider pour la branche</t>
   </si>
   <si>
-    <t>creation de branche, maquette + coder html</t>
+    <t>coder html</t>
+  </si>
+  <si>
+    <t>creation de branche</t>
+  </si>
+  <si>
+    <t>creation de application map</t>
+  </si>
+  <si>
+    <t>apprendre du git</t>
+  </si>
+  <si>
+    <t>jeudi, 15 janvier 2026</t>
+  </si>
+  <si>
+    <t>commencer fenêtre acceuil html</t>
+  </si>
+  <si>
+    <t>encor plus de html</t>
+  </si>
+  <si>
+    <t>faire une application map</t>
   </si>
 </sst>
 </file>
@@ -553,7 +571,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -602,6 +620,9 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1216,13 +1237,13 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>11.25</c:v>
+                  <c:v>11.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>2.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>120.5</c:v>
+                  <c:v>125.75</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>3.25</c:v>
@@ -1945,8 +1966,8 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BDEB89E1-6F36-4738-9369-27FC44324FE7}" name="Tableau1" displayName="Tableau1" ref="A1:F300" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
   <autoFilter ref="A1:F300" xr:uid="{BDEB89E1-6F36-4738-9369-27FC44324FE7}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F1048576">
-    <sortCondition descending="1" ref="D1:D1048576"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F1048575">
+    <sortCondition descending="1" ref="D1:D1048575"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{8F098A10-6760-4DE7-9A95-ADC92EF787A0}" name="Jour" dataDxfId="9"/>
@@ -2282,7 +2303,7 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6">
+      <c r="A2" s="17">
         <v>46034</v>
       </c>
       <c r="B2" s="14">
@@ -2295,12 +2316,12 @@
         <v>7</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F2" s="8"/>
     </row>
     <row r="3" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="6">
+      <c r="A3" s="17">
         <v>46035</v>
       </c>
       <c r="B3" s="14">
@@ -2318,14 +2339,14 @@
       <c r="F3" s="8"/>
     </row>
     <row r="4" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="6">
+      <c r="A4" s="17">
         <v>46036</v>
       </c>
       <c r="B4" s="14">
         <v>1</v>
       </c>
       <c r="C4" s="11">
-        <v>6</v>
+        <v>1.5</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>9</v>
@@ -2334,69 +2355,119 @@
         <v>153</v>
       </c>
       <c r="F4" s="8" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="17">
+        <v>46036</v>
+      </c>
+      <c r="B5" s="14">
+        <v>1</v>
+      </c>
+      <c r="C5" s="11">
+        <v>3.5</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="6"/>
-      <c r="B5" s="14"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="8"/>
       <c r="F5" s="8"/>
     </row>
     <row r="6" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="6"/>
-      <c r="B6" s="14"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="8"/>
+      <c r="A6" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="B6" s="15">
+        <v>1</v>
+      </c>
+      <c r="C6" s="12">
+        <v>1.5</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>155</v>
+      </c>
       <c r="F6" s="8"/>
     </row>
     <row r="7" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="6">
-        <v>46039</v>
+      <c r="A7" s="17">
+        <v>46037</v>
       </c>
       <c r="B7" s="14">
         <v>1</v>
       </c>
       <c r="C7" s="11">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>15</v>
+        <v>154</v>
       </c>
       <c r="F7" s="8"/>
     </row>
     <row r="8" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="6"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="8"/>
+      <c r="A8" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="B8" s="14">
+        <v>1</v>
+      </c>
+      <c r="C8" s="11">
+        <v>0.75</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>157</v>
+      </c>
       <c r="F8" s="8"/>
     </row>
     <row r="9" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="6"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="8"/>
+      <c r="A9" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" s="14">
+        <v>1</v>
+      </c>
+      <c r="C9" s="11">
+        <v>2</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>158</v>
+      </c>
       <c r="F9" s="8"/>
     </row>
     <row r="10" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="6"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="8"/>
+      <c r="A10" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="B10" s="14">
+        <v>1</v>
+      </c>
+      <c r="C10" s="11">
+        <v>2</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>159</v>
+      </c>
       <c r="F10" s="8"/>
     </row>
     <row r="11" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="6"/>
+      <c r="A11" s="17"/>
       <c r="B11" s="14"/>
       <c r="C11" s="11"/>
       <c r="D11" s="7"/>
@@ -2404,7 +2475,7 @@
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="6"/>
+      <c r="A12" s="17"/>
       <c r="B12" s="14"/>
       <c r="C12" s="11"/>
       <c r="D12" s="7"/>
@@ -2412,7 +2483,7 @@
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="6"/>
+      <c r="A13" s="17"/>
       <c r="B13" s="14"/>
       <c r="C13" s="11"/>
       <c r="D13" s="7"/>
@@ -2420,7 +2491,7 @@
       <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="6"/>
+      <c r="A14" s="17"/>
       <c r="B14" s="14"/>
       <c r="C14" s="11"/>
       <c r="D14" s="7"/>
@@ -2428,7 +2499,7 @@
       <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="6"/>
+      <c r="A15" s="17"/>
       <c r="B15" s="14"/>
       <c r="C15" s="11"/>
       <c r="D15" s="7"/>
@@ -2436,7 +2507,7 @@
       <c r="F15" s="8"/>
     </row>
     <row r="16" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="6"/>
+      <c r="A16" s="17"/>
       <c r="B16" s="14"/>
       <c r="C16" s="11"/>
       <c r="D16" s="7"/>
@@ -2444,7 +2515,7 @@
       <c r="F16" s="8"/>
     </row>
     <row r="17" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="6"/>
+      <c r="A17" s="17"/>
       <c r="B17" s="14"/>
       <c r="C17" s="11"/>
       <c r="D17" s="7"/>
@@ -2452,7 +2523,7 @@
       <c r="F17" s="8"/>
     </row>
     <row r="18" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="6"/>
+      <c r="A18" s="17"/>
       <c r="B18" s="14"/>
       <c r="C18" s="11"/>
       <c r="D18" s="7"/>
@@ -2460,7 +2531,7 @@
       <c r="F18" s="8"/>
     </row>
     <row r="19" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="6"/>
+      <c r="A19" s="17"/>
       <c r="B19" s="14"/>
       <c r="C19" s="11"/>
       <c r="D19" s="7"/>
@@ -2468,7 +2539,7 @@
       <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="6"/>
+      <c r="A20" s="17"/>
       <c r="B20" s="14"/>
       <c r="C20" s="11"/>
       <c r="D20" s="7"/>
@@ -2476,7 +2547,7 @@
       <c r="F20" s="8"/>
     </row>
     <row r="21" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="6"/>
+      <c r="A21" s="17"/>
       <c r="B21" s="14"/>
       <c r="C21" s="11"/>
       <c r="D21" s="7"/>
@@ -2484,7 +2555,7 @@
       <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="6"/>
+      <c r="A22" s="17"/>
       <c r="B22" s="14"/>
       <c r="C22" s="11"/>
       <c r="D22" s="7"/>
@@ -2492,7 +2563,7 @@
       <c r="F22" s="8"/>
     </row>
     <row r="23" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="6"/>
+      <c r="A23" s="17"/>
       <c r="B23" s="14"/>
       <c r="C23" s="11"/>
       <c r="D23" s="7"/>
@@ -2500,7 +2571,7 @@
       <c r="F23" s="8"/>
     </row>
     <row r="24" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="6"/>
+      <c r="A24" s="17"/>
       <c r="B24" s="14"/>
       <c r="C24" s="11"/>
       <c r="D24" s="7"/>
@@ -2577,7 +2648,7 @@
         <v>7</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F32" s="8"/>
     </row>
@@ -2595,7 +2666,7 @@
         <v>7</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F33" s="8"/>
     </row>
@@ -2613,7 +2684,7 @@
         <v>7</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F34" s="8"/>
     </row>
@@ -2631,7 +2702,7 @@
         <v>8</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F35" s="8"/>
     </row>
@@ -2649,7 +2720,7 @@
         <v>11</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F36" s="8"/>
     </row>
@@ -2667,7 +2738,7 @@
         <v>11</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F37" s="8"/>
     </row>
@@ -2685,7 +2756,7 @@
         <v>11</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F38" s="8"/>
     </row>
@@ -2703,7 +2774,7 @@
         <v>11</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F39" s="8"/>
     </row>
@@ -2721,7 +2792,7 @@
         <v>9</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F40" s="8"/>
     </row>
@@ -2739,10 +2810,10 @@
         <v>9</v>
       </c>
       <c r="E41" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="F41" s="8" t="s">
         <v>27</v>
-      </c>
-      <c r="F41" s="8" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2759,7 +2830,7 @@
         <v>9</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F42" s="8"/>
     </row>
@@ -2777,7 +2848,7 @@
         <v>9</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F43" s="8"/>
     </row>
@@ -2795,7 +2866,7 @@
         <v>9</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F44" s="8"/>
     </row>
@@ -2813,7 +2884,7 @@
         <v>9</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F45" s="8"/>
     </row>
@@ -2831,7 +2902,7 @@
         <v>9</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F46" s="8"/>
     </row>
@@ -2849,7 +2920,7 @@
         <v>9</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F47" s="8"/>
     </row>
@@ -2867,7 +2938,7 @@
         <v>9</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F48" s="8"/>
     </row>
@@ -2885,7 +2956,7 @@
         <v>9</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F49" s="8"/>
     </row>
@@ -2903,7 +2974,7 @@
         <v>9</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F50" s="8"/>
     </row>
@@ -2921,7 +2992,7 @@
         <v>9</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F51" s="8"/>
     </row>
@@ -2939,7 +3010,7 @@
         <v>6</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F52" s="8"/>
     </row>
@@ -2957,7 +3028,7 @@
         <v>9</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F53" s="8"/>
     </row>
@@ -2975,10 +3046,10 @@
         <v>9</v>
       </c>
       <c r="E54" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="F54" s="8" t="s">
         <v>41</v>
-      </c>
-      <c r="F54" s="8" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2995,7 +3066,7 @@
         <v>9</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F55" s="8"/>
     </row>
@@ -3013,7 +3084,7 @@
         <v>9</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F56" s="8"/>
     </row>
@@ -3031,7 +3102,7 @@
         <v>9</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F57" s="8"/>
     </row>
@@ -3049,7 +3120,7 @@
         <v>9</v>
       </c>
       <c r="E58" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F58" s="8"/>
     </row>
@@ -3067,7 +3138,7 @@
         <v>9</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F59" s="8"/>
     </row>
@@ -3085,7 +3156,7 @@
         <v>9</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F60" s="8"/>
     </row>
@@ -3103,10 +3174,10 @@
         <v>9</v>
       </c>
       <c r="E61" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="F61" s="8" t="s">
         <v>49</v>
-      </c>
-      <c r="F61" s="8" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3123,7 +3194,7 @@
         <v>6</v>
       </c>
       <c r="E62" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F62" s="8"/>
     </row>
@@ -3141,7 +3212,7 @@
         <v>9</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F63" s="8"/>
     </row>
@@ -3159,10 +3230,10 @@
         <v>9</v>
       </c>
       <c r="E64" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F64" s="8" t="s">
         <v>52</v>
-      </c>
-      <c r="F64" s="8" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3179,7 +3250,7 @@
         <v>9</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F65" s="8"/>
     </row>
@@ -3197,7 +3268,7 @@
         <v>9</v>
       </c>
       <c r="E66" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F66" s="8"/>
     </row>
@@ -3215,7 +3286,7 @@
         <v>9</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F67" s="8"/>
     </row>
@@ -3233,10 +3304,10 @@
         <v>9</v>
       </c>
       <c r="E68" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="F68" s="8" t="s">
         <v>57</v>
-      </c>
-      <c r="F68" s="8" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3253,7 +3324,7 @@
         <v>11</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F69" s="8"/>
     </row>
@@ -3271,7 +3342,7 @@
         <v>6</v>
       </c>
       <c r="E70" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F70" s="8"/>
     </row>
@@ -3289,10 +3360,10 @@
         <v>9</v>
       </c>
       <c r="E71" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="F71" s="8" t="s">
         <v>60</v>
-      </c>
-      <c r="F71" s="8" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3309,10 +3380,10 @@
         <v>9</v>
       </c>
       <c r="E72" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F72" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3329,7 +3400,7 @@
         <v>9</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F73" s="8"/>
     </row>
@@ -3347,10 +3418,10 @@
         <v>9</v>
       </c>
       <c r="E74" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="F74" s="8" t="s">
         <v>64</v>
-      </c>
-      <c r="F74" s="8" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="75" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3367,7 +3438,7 @@
         <v>9</v>
       </c>
       <c r="E75" s="8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F75" s="8"/>
     </row>
@@ -3385,7 +3456,7 @@
         <v>9</v>
       </c>
       <c r="E76" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F76" s="8"/>
     </row>
@@ -3403,10 +3474,10 @@
         <v>9</v>
       </c>
       <c r="E77" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="F77" s="8" t="s">
         <v>68</v>
-      </c>
-      <c r="F77" s="8" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="78" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3423,7 +3494,7 @@
         <v>6</v>
       </c>
       <c r="E78" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F78" s="8"/>
     </row>
@@ -3441,10 +3512,10 @@
         <v>9</v>
       </c>
       <c r="E79" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="F79" s="8" t="s">
         <v>70</v>
-      </c>
-      <c r="F79" s="8" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="80" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3461,10 +3532,10 @@
         <v>9</v>
       </c>
       <c r="E80" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F80" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="81" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3481,7 +3552,7 @@
         <v>9</v>
       </c>
       <c r="E81" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F81" s="8"/>
     </row>
@@ -3499,10 +3570,10 @@
         <v>9</v>
       </c>
       <c r="E82" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F82" s="8" t="s">
         <v>74</v>
-      </c>
-      <c r="F82" s="8" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="83" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3519,7 +3590,7 @@
         <v>11</v>
       </c>
       <c r="E83" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F83" s="8"/>
     </row>
@@ -3537,7 +3608,7 @@
         <v>11</v>
       </c>
       <c r="E84" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F84" s="8"/>
     </row>
@@ -3555,7 +3626,7 @@
         <v>11</v>
       </c>
       <c r="E85" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F85" s="8"/>
     </row>
@@ -3573,7 +3644,7 @@
         <v>11</v>
       </c>
       <c r="E86" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F86" s="8"/>
     </row>
@@ -3591,7 +3662,7 @@
         <v>6</v>
       </c>
       <c r="E87" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F87" s="8"/>
     </row>
@@ -3609,10 +3680,10 @@
         <v>6</v>
       </c>
       <c r="E88" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F88" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="89" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3629,7 +3700,7 @@
         <v>11</v>
       </c>
       <c r="E89" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F89" s="8"/>
     </row>
@@ -3647,7 +3718,7 @@
         <v>9</v>
       </c>
       <c r="E90" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F90" s="8"/>
     </row>
@@ -3665,7 +3736,7 @@
         <v>6</v>
       </c>
       <c r="E91" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F91" s="8"/>
     </row>
@@ -3683,7 +3754,7 @@
         <v>6</v>
       </c>
       <c r="E92" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F92" s="8"/>
     </row>
@@ -3701,7 +3772,7 @@
         <v>9</v>
       </c>
       <c r="E93" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F93" s="8"/>
     </row>
@@ -3719,10 +3790,10 @@
         <v>9</v>
       </c>
       <c r="E94" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="F94" s="8" t="s">
         <v>85</v>
-      </c>
-      <c r="F94" s="8" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="95" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3739,7 +3810,7 @@
         <v>9</v>
       </c>
       <c r="E95" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F95" s="8"/>
     </row>
@@ -3757,10 +3828,10 @@
         <v>9</v>
       </c>
       <c r="E96" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="F96" s="8" t="s">
         <v>88</v>
-      </c>
-      <c r="F96" s="8" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="97" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3777,7 +3848,7 @@
         <v>9</v>
       </c>
       <c r="E97" s="8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F97" s="8"/>
     </row>
@@ -3795,10 +3866,10 @@
         <v>9</v>
       </c>
       <c r="E98" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="F98" s="8" t="s">
         <v>90</v>
-      </c>
-      <c r="F98" s="8" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="99" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3815,7 +3886,7 @@
         <v>9</v>
       </c>
       <c r="E99" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F99" s="8"/>
     </row>
@@ -3833,7 +3904,7 @@
         <v>9</v>
       </c>
       <c r="E100" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F100" s="8"/>
     </row>
@@ -3851,7 +3922,7 @@
         <v>9</v>
       </c>
       <c r="E101" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F101" s="8"/>
     </row>
@@ -3869,7 +3940,7 @@
         <v>9</v>
       </c>
       <c r="E102" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F102" s="8"/>
     </row>
@@ -3887,7 +3958,7 @@
         <v>9</v>
       </c>
       <c r="E103" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F103" s="8"/>
     </row>
@@ -3905,7 +3976,7 @@
         <v>9</v>
       </c>
       <c r="E104" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F104" s="8"/>
     </row>
@@ -3923,7 +3994,7 @@
         <v>6</v>
       </c>
       <c r="E105" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F105" s="8"/>
     </row>
@@ -3941,7 +4012,7 @@
         <v>9</v>
       </c>
       <c r="E106" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F106" s="8"/>
     </row>
@@ -3959,7 +4030,7 @@
         <v>9</v>
       </c>
       <c r="E107" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F107" s="8"/>
     </row>
@@ -3977,7 +4048,7 @@
         <v>9</v>
       </c>
       <c r="E108" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F108" s="8"/>
     </row>
@@ -3995,10 +4066,10 @@
         <v>9</v>
       </c>
       <c r="E109" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="F109" s="8" t="s">
         <v>102</v>
-      </c>
-      <c r="F109" s="8" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="110" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4015,10 +4086,10 @@
         <v>9</v>
       </c>
       <c r="E110" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="F110" s="8" t="s">
         <v>104</v>
-      </c>
-      <c r="F110" s="8" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="111" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4035,7 +4106,7 @@
         <v>9</v>
       </c>
       <c r="E111" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F111" s="8"/>
     </row>
@@ -4053,7 +4124,7 @@
         <v>9</v>
       </c>
       <c r="E112" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F112" s="8"/>
     </row>
@@ -4071,7 +4142,7 @@
         <v>9</v>
       </c>
       <c r="E113" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F113" s="8"/>
     </row>
@@ -4089,7 +4160,7 @@
         <v>9</v>
       </c>
       <c r="E114" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F114" s="8"/>
     </row>
@@ -4107,10 +4178,10 @@
         <v>9</v>
       </c>
       <c r="E115" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="F115" s="8" t="s">
         <v>110</v>
-      </c>
-      <c r="F115" s="8" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="116" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4127,7 +4198,7 @@
         <v>9</v>
       </c>
       <c r="E116" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F116" s="8"/>
     </row>
@@ -4145,7 +4216,7 @@
         <v>9</v>
       </c>
       <c r="E117" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F117" s="8"/>
     </row>
@@ -4163,7 +4234,7 @@
         <v>9</v>
       </c>
       <c r="E118" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F118" s="8"/>
     </row>
@@ -4181,7 +4252,7 @@
         <v>9</v>
       </c>
       <c r="E119" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F119" s="8"/>
     </row>
@@ -4199,7 +4270,7 @@
         <v>9</v>
       </c>
       <c r="E120" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F120" s="8"/>
     </row>
@@ -4217,7 +4288,7 @@
         <v>9</v>
       </c>
       <c r="E121" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F121" s="8"/>
     </row>
@@ -4235,7 +4306,7 @@
         <v>9</v>
       </c>
       <c r="E122" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F122" s="8"/>
     </row>
@@ -4253,7 +4324,7 @@
         <v>9</v>
       </c>
       <c r="E123" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F123" s="8"/>
     </row>
@@ -4271,7 +4342,7 @@
         <v>6</v>
       </c>
       <c r="E124" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F124" s="8"/>
     </row>
@@ -4289,7 +4360,7 @@
         <v>6</v>
       </c>
       <c r="E125" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F125" s="8"/>
     </row>
@@ -4307,10 +4378,10 @@
         <v>9</v>
       </c>
       <c r="E126" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="F126" s="8" t="s">
         <v>121</v>
-      </c>
-      <c r="F126" s="8" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="127" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4327,7 +4398,7 @@
         <v>9</v>
       </c>
       <c r="E127" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F127" s="8"/>
     </row>
@@ -4345,7 +4416,7 @@
         <v>9</v>
       </c>
       <c r="E128" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F128" s="8"/>
     </row>
@@ -4363,7 +4434,7 @@
         <v>9</v>
       </c>
       <c r="E129" s="8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F129" s="8"/>
     </row>
@@ -4381,7 +4452,7 @@
         <v>9</v>
       </c>
       <c r="E130" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F130" s="8"/>
     </row>
@@ -4399,7 +4470,7 @@
         <v>10</v>
       </c>
       <c r="E131" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F131" s="8"/>
     </row>
@@ -4417,7 +4488,7 @@
         <v>10</v>
       </c>
       <c r="E132" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F132" s="8"/>
     </row>
@@ -4435,7 +4506,7 @@
         <v>6</v>
       </c>
       <c r="E133" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F133" s="8"/>
     </row>
@@ -4453,10 +4524,10 @@
         <v>9</v>
       </c>
       <c r="E134" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="F134" s="8" t="s">
         <v>130</v>
-      </c>
-      <c r="F134" s="8" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="135" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4473,10 +4544,10 @@
         <v>10</v>
       </c>
       <c r="E135" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F135" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="136" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4493,7 +4564,7 @@
         <v>6</v>
       </c>
       <c r="E136" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F136" s="8"/>
     </row>
@@ -4511,7 +4582,7 @@
         <v>6</v>
       </c>
       <c r="E137" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F137" s="8"/>
     </row>
@@ -4529,7 +4600,7 @@
         <v>9</v>
       </c>
       <c r="E138" s="8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F138" s="8"/>
     </row>
@@ -4547,7 +4618,7 @@
         <v>9</v>
       </c>
       <c r="E139" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F139" s="8"/>
     </row>
@@ -4565,7 +4636,7 @@
         <v>9</v>
       </c>
       <c r="E140" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F140" s="8"/>
     </row>
@@ -4583,7 +4654,7 @@
         <v>11</v>
       </c>
       <c r="E141" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F141" s="8"/>
     </row>
@@ -4601,7 +4672,7 @@
         <v>11</v>
       </c>
       <c r="E142" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F142" s="8"/>
     </row>
@@ -4619,7 +4690,7 @@
         <v>11</v>
       </c>
       <c r="E143" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F143" s="8"/>
     </row>
@@ -4637,7 +4708,7 @@
         <v>6</v>
       </c>
       <c r="E144" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F144" s="8"/>
     </row>
@@ -4655,7 +4726,7 @@
         <v>11</v>
       </c>
       <c r="E145" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F145" s="8"/>
     </row>
@@ -4673,7 +4744,7 @@
         <v>11</v>
       </c>
       <c r="E146" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F146" s="8"/>
     </row>
@@ -4691,7 +4762,7 @@
         <v>11</v>
       </c>
       <c r="E147" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F147" s="8"/>
     </row>
@@ -4709,7 +4780,7 @@
         <v>6</v>
       </c>
       <c r="E148" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F148" s="8"/>
     </row>
@@ -4727,7 +4798,7 @@
         <v>6</v>
       </c>
       <c r="E149" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F149" s="8"/>
     </row>
@@ -4745,7 +4816,7 @@
         <v>11</v>
       </c>
       <c r="E150" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F150" s="8"/>
     </row>
@@ -4763,7 +4834,7 @@
         <v>11</v>
       </c>
       <c r="E151" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F151" s="8"/>
     </row>
@@ -4781,7 +4852,7 @@
         <v>11</v>
       </c>
       <c r="E152" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F152" s="8"/>
     </row>
@@ -4799,7 +4870,7 @@
         <v>11</v>
       </c>
       <c r="E153" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F153" s="8"/>
     </row>
@@ -4817,7 +4888,7 @@
         <v>6</v>
       </c>
       <c r="E154" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F154" s="8"/>
     </row>
@@ -4835,7 +4906,7 @@
         <v>9</v>
       </c>
       <c r="E155" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F155" s="8"/>
     </row>
@@ -4853,7 +4924,7 @@
         <v>11</v>
       </c>
       <c r="E156" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F156" s="8"/>
     </row>
@@ -4871,7 +4942,7 @@
         <v>11</v>
       </c>
       <c r="E157" s="8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F157" s="8"/>
     </row>
@@ -4889,7 +4960,7 @@
         <v>6</v>
       </c>
       <c r="E158" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F158" s="8"/>
     </row>
@@ -4907,7 +4978,7 @@
         <v>6</v>
       </c>
       <c r="E159" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F159" s="8"/>
     </row>
@@ -4925,7 +4996,7 @@
         <v>11</v>
       </c>
       <c r="E160" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F160" s="8"/>
     </row>
@@ -7651,11 +7722,11 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B300" xr:uid="{E1FCDE41-ACF1-4A68-9483-C062BB428146}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7:B300 B1:B5" xr:uid="{E1FCDE41-ACF1-4A68-9483-C062BB428146}">
       <formula1>1</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C300" xr:uid="{48106778-5E48-49BE-9E53-EB975C533ABF}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C300 C1:C5" xr:uid="{48106778-5E48-49BE-9E53-EB975C533ABF}">
       <formula1>0.25</formula1>
       <formula2>10</formula2>
     </dataValidation>
@@ -7675,7 +7746,7 @@
           <x14:formula1>
             <xm:f>Listes!$A:$A</xm:f>
           </x14:formula1>
-          <xm:sqref>D1:D300</xm:sqref>
+          <xm:sqref>D7:D300 D1:D5</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -7706,7 +7777,7 @@
       </c>
       <c r="B2" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>11.25</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -7724,7 +7795,7 @@
       </c>
       <c r="B4" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>120.5</v>
+        <v>125.75</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
docs:: update the journal
</commit_message>
<xml_diff>
--- a/Annexes/Journal_de_travail/Journal_de_Travail_Léonard_Weber.xlsx
+++ b/Annexes/Journal_de_travail/Journal_de_Travail_Léonard_Weber.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduvaud-my.sharepoint.com/personal/pe04cuw_eduvaud_ch/Documents/CPNV_2025-2026/Semaine.projet.lego/journal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="362" documentId="13_ncr:1_{EFDCB34D-4D99-487E-82C9-6E7A8D14F32E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD85DE2C-997A-49C3-A803-5A211CE6396E}"/>
+  <xr:revisionPtr revIDLastSave="706" documentId="13_ncr:1_{EFDCB34D-4D99-487E-82C9-6E7A8D14F32E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8AD77C54-DF8B-477E-BE2F-D1D88DB0736F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="Stats" sheetId="5" r:id="rId3"/>
     <sheet name="Listes" sheetId="2" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="61">
   <si>
     <t>Jour</t>
   </si>
@@ -92,349 +92,10 @@
     <t>Sprint Review avec le CdP</t>
   </si>
   <si>
-    <t>Re-schématisation des use cases</t>
-  </si>
-  <si>
-    <t>Ajout de spécifications dans les scénarios</t>
-  </si>
-  <si>
-    <t>Modification du MCD</t>
-  </si>
-  <si>
-    <t>Modification du MLD</t>
-  </si>
-  <si>
-    <t>Documentation - Modification de l'introduction</t>
-  </si>
-  <si>
-    <t>Documentation - Mise à jour d'images</t>
-  </si>
-  <si>
-    <t>Documentation - Ajout d'un paragraphe a la stratégie de tests</t>
-  </si>
-  <si>
-    <t>Mise en forme</t>
-  </si>
-  <si>
-    <t>Création d'une page d'acceuil</t>
-  </si>
-  <si>
-    <t>Modification du gabarit</t>
-  </si>
-  <si>
-    <t>Gabarit est maintenant repoonsive et dynamique en fonction d'un guest ou user</t>
-  </si>
-  <si>
-    <t>Ajout du fichier dbconnector</t>
-  </si>
-  <si>
-    <t>Création de la vue 'register'</t>
-  </si>
-  <si>
-    <t>Liaison de la fonction register avec la BDD</t>
-  </si>
-  <si>
-    <t>Gestion des erreurs liées au register</t>
-  </si>
-  <si>
-    <t>Création de la vue 'login'</t>
-  </si>
-  <si>
-    <t>Liaison de la fonction login avec la BDD</t>
-  </si>
-  <si>
-    <t>Gestion des erreurs liées au login</t>
-  </si>
-  <si>
-    <t>Ajout du logout</t>
-  </si>
-  <si>
-    <t>Création de la vue 'locations'</t>
-  </si>
-  <si>
-    <t>Dynamisation de la vue 'locations'</t>
-  </si>
-  <si>
-    <t>Commits github et journal de travail</t>
-  </si>
-  <si>
-    <t>Création de la vue 'specificLocation'</t>
-  </si>
-  <si>
-    <t>Recherches pour l'ajout d'un datepicker à la vue 'specificLocation'</t>
-  </si>
-  <si>
-    <t>Le datepicker devait avoir pour caractéristique de pouvoir désactiver des dates bien précises.</t>
-  </si>
-  <si>
-    <t>Ajout du datepicker</t>
-  </si>
-  <si>
-    <t>Dynamisation de la vue 'specificLocation'</t>
-  </si>
-  <si>
-    <t>Dynamisation du datepicker</t>
-  </si>
-  <si>
-    <t>Ajout d'un carousel si la location contient plus d'une image</t>
-  </si>
-  <si>
-    <t>Ajout de la fonctionnalité de recherche</t>
-  </si>
-  <si>
-    <t>Création d'un formulaire de recherche avancée</t>
-  </si>
-  <si>
-    <t>Configuration des datepicker du formulaire de recherche</t>
-  </si>
-  <si>
-    <t>Le formulaire contenant une date de début et une date de fin, je me suis assuré que le datepicker de fin ne puisse pas contenir une date précédent la date de début.</t>
-  </si>
-  <si>
-    <t>Création d'une fonction sql dynamique en fonction des paramètres utilisés pour le filtrage</t>
-  </si>
-  <si>
-    <t>Création de la fonction de filtrage dans le controller</t>
-  </si>
-  <si>
-    <t>Difficultés à vérifier que les dates séléctionnées dans le formulaire de filtrage ne sont pas comprises dans les locations renvoyées par la BDD</t>
-  </si>
-  <si>
-    <t>Création de la vue permettant aux utilisateurs d'ajouter/modifier une location</t>
-  </si>
-  <si>
-    <t>Création du formulaire d'ajout de location</t>
-  </si>
-  <si>
-    <t>Ajout de boutons au formulaire d'ajout de location afin d'ajouter / supprimer un champ image</t>
-  </si>
-  <si>
-    <t>Fonction d'ajout de location dans le controller</t>
-  </si>
-  <si>
-    <t>Récupère correctement toutes les données et intégre l'image dans les fichiers du projet mais ne fait pas encore le lien avec la BDD</t>
-  </si>
-  <si>
-    <t>Documentation - Planification</t>
-  </si>
-  <si>
-    <t>Ajout d'une fonction de génération de n° de série</t>
-  </si>
-  <si>
-    <t>Sert à générer les n° de locations et de réservations</t>
-  </si>
-  <si>
-    <t>Insère maintenant également les données dans la BDD (location + images) et traite les erreurs</t>
-  </si>
-  <si>
-    <t>Création d'une vue permettant de choisir une location à modifier</t>
-  </si>
-  <si>
-    <t>Tentatives d'améliorations de la vue du choix de location à modifier (abandon)</t>
-  </si>
-  <si>
-    <t>Je voulais ajouter un champ contenant le nom de la location afin de donner plus d'informations à l'utilisateurs mais je n'ai pas voulu y sacrifier trop de temps pour le moment</t>
-  </si>
-  <si>
-    <t>Création d'une vue contenant un formulaire de modification de location</t>
-  </si>
-  <si>
-    <t>Gestion des inputs d'image du formulaire de modification de location</t>
-  </si>
-  <si>
-    <t>Fonction de modification de locations dans le controller</t>
-  </si>
-  <si>
-    <t>Gestion des erreurs d'inputs + Ajout d'images au projet</t>
-  </si>
-  <si>
-    <t>Modification de la vue contenant le formulaire de modification de location</t>
-  </si>
-  <si>
-    <t>Ajout d'un input de type hidden afin de stocker les valeurs des anciennes images à supprimer. Temps perdu sur la fonction js</t>
-  </si>
-  <si>
-    <t>Suppressions des images dans le projet, gestion des images dand la BDD, modfication de la location dans la BDD</t>
-  </si>
-  <si>
-    <t>Ajout de la fonctionnalité de suppresion de locations</t>
-  </si>
-  <si>
-    <t>Ajout d'en-têtes / commentaires de manière globale</t>
-  </si>
-  <si>
-    <t>J'avais oublié de le faire depuis un petit moment</t>
-  </si>
-  <si>
-    <t>Documentation - Répertoire de projet</t>
-  </si>
-  <si>
-    <t>Documentation - Architecture du projet</t>
-  </si>
-  <si>
-    <t>Documentation - Script BDD</t>
-  </si>
-  <si>
-    <t>Documentation - Algorithme de chiffrement</t>
-  </si>
-  <si>
-    <t>Visite du deuxième expert M. Girardet</t>
-  </si>
-  <si>
-    <t>Dernières mini modifications à faire sur la phase d'analyse et discussion sur l'avancée du projet etc…</t>
-  </si>
-  <si>
-    <t>Réorganisation des fichiers de dév</t>
-  </si>
-  <si>
-    <t>Préparation des documents et du mail nécessaires au rendu</t>
-  </si>
-  <si>
-    <t>Création d'une vue pour la réservation de locations</t>
-  </si>
-  <si>
-    <t>Configuration des datepicker de la vue de réservation</t>
-  </si>
-  <si>
-    <t>Désactivent les dates avant aujourd'hui, dates déjà réservées et impossibilité d'avoir une date de fin avant la date de début</t>
-  </si>
-  <si>
-    <t>Affichage du prix en fonction des dates prévues</t>
-  </si>
-  <si>
-    <t>Réalisation de la fonction de réservation de locations</t>
-  </si>
-  <si>
-    <t>Traitement des données + ajout à la BDD</t>
-  </si>
-  <si>
-    <t>Configuration de swisscenter</t>
-  </si>
-  <si>
-    <t>Erreurs, BDD</t>
-  </si>
-  <si>
-    <t>Ajout de PHPMailer au projet</t>
-  </si>
-  <si>
-    <t>Création d'une adresse mail sur swisscenter</t>
-  </si>
-  <si>
-    <t>Mise en place de la connexion entre code et serveur SMTP</t>
-  </si>
-  <si>
-    <t>Réalisation du mail de confirmation à l'utilisateur</t>
-  </si>
-  <si>
-    <t>Réalisation du mail de confirmation au loueur</t>
-  </si>
-  <si>
-    <t>Adaptations du code pour la version en ligne</t>
-  </si>
-  <si>
-    <t>Oubli du JdT + Commits GitHub --&gt; Réalisation le 23.05.2023</t>
-  </si>
-  <si>
-    <t>Création d'une vue pour le menu administrateur</t>
-  </si>
-  <si>
-    <t>Création d'une vue pour le menu de gestion des utilisateurs</t>
-  </si>
-  <si>
-    <t>Liaison entre le menu admin et le menu de gestion des utilisateurs</t>
-  </si>
-  <si>
-    <t>Création d'une vue contenant un formulaire d'ajout d'utilisateurs</t>
-  </si>
-  <si>
-    <t>Reprise du formulaire de register</t>
-  </si>
-  <si>
-    <t>Réalisation de la fonction d'ajout d'utilisateurs</t>
-  </si>
-  <si>
-    <t>Amélioration possible en fusionnant la fonction avec celle du register</t>
-  </si>
-  <si>
-    <t>Création d'une vue permettant de choisir un utilisateur à modifier</t>
-  </si>
-  <si>
-    <t>Création d'une vue contenant un formulaire de modification / suppression d'utilisateurs</t>
-  </si>
-  <si>
-    <t>Réalisation de la fonction de modification d'utilisateurs</t>
-  </si>
-  <si>
-    <t>Réalisation de la fonction de suppression d'utilisateurs</t>
-  </si>
-  <si>
-    <t>Création d'une vue pour le menu de gestion des locations</t>
-  </si>
-  <si>
-    <t>Réalisation des fonction CRUD quant aux locations plus rapide que prévu car elles avaient déjà été effectuée d'un point de vue d'utilisateur. Une amélioration pourrait cepandant être mise en place car le code est donc quasiment à "double". Il faudrait donc fusionner les fonctions des deux points de vue en une seule fonction</t>
-  </si>
-  <si>
-    <t>Liaison entre le menu admin et le menu de gestion des locations</t>
-  </si>
-  <si>
-    <t>Création d'une vue contenant un formulaire d'ajout de locations</t>
-  </si>
-  <si>
-    <t>Réalisation de la fonction d'ajout de locations</t>
-  </si>
-  <si>
-    <t>Création d'une vue contenant un formulaire de modification / suppression de  locations</t>
-  </si>
-  <si>
-    <t>Réalisation de la fonction de modification de locations</t>
-  </si>
-  <si>
-    <t>Réalisation de la fonction de suppression de locations</t>
-  </si>
-  <si>
-    <t>Débug du code suite à des erreurs présentes sur la version en ligne</t>
-  </si>
-  <si>
-    <t>JdT + Commits GitHub de la veille + aujourd'hui</t>
-  </si>
-  <si>
-    <t>Préparation des documents et mail nécessaire au rendu</t>
-  </si>
-  <si>
-    <t>Résolution de problèmes de CSS</t>
-  </si>
-  <si>
-    <t>Ajout d'un deuxième fichier css par tailwind plus "propre" et organisé</t>
-  </si>
-  <si>
-    <t>Ajout d'un carousel dynamique sur la page d'acceuil</t>
-  </si>
-  <si>
-    <t>Gestion des taille d'images dans la page d'acceuil et dans la page contenant les locations</t>
-  </si>
-  <si>
     <t>Gestion d'erreurs supplémentaires dans les formulaires</t>
   </si>
   <si>
-    <t>Améliorations et debug général</t>
-  </si>
-  <si>
-    <t>Choix des tests à effectuer</t>
-  </si>
-  <si>
-    <t>Réalisation de tests</t>
-  </si>
-  <si>
     <t>Commits GitHub + JdT</t>
-  </si>
-  <si>
-    <t>Observation d'un problème avec SwissCenter et tentatives de résolution</t>
-  </si>
-  <si>
-    <t>Durant la nuit, l'entiereté du projet a été supprimé sur SwissCenter pour une raison que j'ignore. J'ai tenté d'utiliser une backup afin de restaurer le site mais PHP ne semble plus fonctionner malgré que la configuration n'a pas changé</t>
-  </si>
-  <si>
-    <t>Tests effectués en local comme la version en ligne ne fonctionne plus</t>
   </si>
   <si>
     <t>Préparation du mail de rendu hebodmadaire</t>
@@ -488,9 +149,6 @@
     <t>Préparation du mail de rendu final</t>
   </si>
   <si>
-    <t>Réalisation du projet sur swisscenter</t>
-  </si>
-  <si>
     <t xml:space="preserve">Découverte du Cahier des charges et organisation </t>
   </si>
   <si>
@@ -515,10 +173,55 @@
     <t>commencer fenêtre acceuil html</t>
   </si>
   <si>
-    <t>encor plus de html</t>
+    <t>faire une application map</t>
   </si>
   <si>
-    <t>faire une application map</t>
+    <t>vendredi, 16 janvier 2026</t>
+  </si>
+  <si>
+    <t>finir application map</t>
+  </si>
+  <si>
+    <t>avec le fichier de que m'a donné édis</t>
+  </si>
+  <si>
+    <t>faie du html ajouter du menu</t>
+  </si>
+  <si>
+    <t>meeting avec le group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mise à jour de application map </t>
+  </si>
+  <si>
+    <t>dans le balsamiq</t>
+  </si>
+  <si>
+    <t xml:space="preserve">regarder vidéo </t>
+  </si>
+  <si>
+    <t>la vidéo explique les application map</t>
+  </si>
+  <si>
+    <t>fini l'appliction map</t>
+  </si>
+  <si>
+    <t>Lundi, 19 janvier 2026</t>
+  </si>
+  <si>
+    <t>user flow de admin</t>
+  </si>
+  <si>
+    <t>Mardi, 20 janvier 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rendez vous avec groupe </t>
+  </si>
+  <si>
+    <t>parler de différente problem / organisation</t>
+  </si>
+  <si>
+    <t>trouver un template/code couleur pour le site</t>
   </si>
 </sst>
 </file>
@@ -528,7 +231,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -546,6 +249,12 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Century Gothic"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Century Gothic"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1237,28 +946,28 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>11.5</c:v>
+                  <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.5</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>125.75</c:v>
+                  <c:v>12.75</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.25</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>35</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>28.75</c:v>
+                  <c:v>1.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>2.25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1930,7 +1639,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="7734300" cy="5035550"/>
+    <xdr:ext cx="9286875" cy="6048375"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Graphique 1">
@@ -2316,7 +2025,7 @@
         <v>7</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>150</v>
+        <v>36</v>
       </c>
       <c r="F2" s="8"/>
     </row>
@@ -2352,10 +2061,10 @@
         <v>9</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>153</v>
+        <v>39</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>151</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2372,13 +2081,13 @@
         <v>9</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>152</v>
+        <v>38</v>
       </c>
       <c r="F5" s="8"/>
     </row>
     <row r="6" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="17" t="s">
-        <v>156</v>
+        <v>42</v>
       </c>
       <c r="B6" s="15">
         <v>1</v>
@@ -2390,7 +2099,7 @@
         <v>7</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>155</v>
+        <v>41</v>
       </c>
       <c r="F6" s="8"/>
     </row>
@@ -2408,13 +2117,13 @@
         <v>9</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>154</v>
+        <v>40</v>
       </c>
       <c r="F7" s="8"/>
     </row>
     <row r="8" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="17" t="s">
-        <v>156</v>
+        <v>42</v>
       </c>
       <c r="B8" s="14">
         <v>1</v>
@@ -2426,13 +2135,13 @@
         <v>9</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>157</v>
+        <v>43</v>
       </c>
       <c r="F8" s="8"/>
     </row>
     <row r="9" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
-        <v>156</v>
+        <v>42</v>
       </c>
       <c r="B9" s="14">
         <v>1</v>
@@ -2444,13 +2153,13 @@
         <v>9</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>158</v>
+        <v>48</v>
       </c>
       <c r="F9" s="8"/>
     </row>
     <row r="10" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="17" t="s">
-        <v>156</v>
+        <v>42</v>
       </c>
       <c r="B10" s="14">
         <v>1</v>
@@ -2459,83 +2168,181 @@
         <v>2</v>
       </c>
       <c r="D10" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F10" s="8"/>
+    </row>
+    <row r="11" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="14">
+        <v>1</v>
+      </c>
+      <c r="C11" s="11">
+        <v>1</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" s="8"/>
+    </row>
+    <row r="12" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" s="14">
+        <v>1</v>
+      </c>
+      <c r="C12" s="11">
+        <v>0.75</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="14">
+        <v>1</v>
+      </c>
+      <c r="C13" s="11">
+        <v>1.5</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="F13" s="8"/>
+    </row>
+    <row r="14" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="14">
+        <v>1</v>
+      </c>
+      <c r="C14" s="11">
+        <v>0.25</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" s="14">
+        <v>1</v>
+      </c>
+      <c r="C15" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="F10" s="8"/>
-    </row>
-    <row r="11" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="17"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-    </row>
-    <row r="12" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="17"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-    </row>
-    <row r="13" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="17"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-    </row>
-    <row r="14" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="17"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-    </row>
-    <row r="15" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="17"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
+      <c r="E15" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="16" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="17"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="8"/>
+      <c r="A16" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="14">
+        <v>1</v>
+      </c>
+      <c r="C16" s="11">
+        <v>2.25</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>54</v>
+      </c>
       <c r="F16" s="8"/>
     </row>
     <row r="17" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="17"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="8"/>
+      <c r="A17" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="B17" s="14">
+        <v>2</v>
+      </c>
+      <c r="C17" s="11">
+        <v>0.75</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>56</v>
+      </c>
       <c r="F17" s="8"/>
     </row>
     <row r="18" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="17"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
+      <c r="A18" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" s="14">
+        <v>2</v>
+      </c>
+      <c r="C18" s="11">
+        <v>1.5</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="19" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="17"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="8"/>
+      <c r="A19" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B19" s="14">
+        <v>2</v>
+      </c>
+      <c r="C19" s="11">
+        <v>0.75</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>60</v>
+      </c>
       <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2635,2368 +2442,1084 @@
       <c r="F31" s="8"/>
     </row>
     <row r="32" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="6">
-        <v>46043</v>
-      </c>
-      <c r="B32" s="14">
-        <v>2</v>
-      </c>
-      <c r="C32" s="11">
-        <v>1.25</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E32" s="8" t="s">
+      <c r="A32" s="6"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="11"/>
+      <c r="D32" s="7"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+    </row>
+    <row r="33" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="6"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="11"/>
+      <c r="D33" s="7"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+    </row>
+    <row r="34" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="6"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="11"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+    </row>
+    <row r="35" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="6"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="11"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+    </row>
+    <row r="36" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="6"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="7"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+    </row>
+    <row r="37" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="6"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="11"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+    </row>
+    <row r="38" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="6"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="11"/>
+      <c r="D38" s="7"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+    </row>
+    <row r="39" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="6"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="11"/>
+      <c r="D39" s="7"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+    </row>
+    <row r="40" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="6"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="11"/>
+      <c r="D40" s="7"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
+    </row>
+    <row r="41" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="6"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="11"/>
+      <c r="D41" s="7"/>
+      <c r="E41" s="8"/>
+      <c r="F41" s="8"/>
+    </row>
+    <row r="42" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="6"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="11"/>
+      <c r="D42" s="7"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="8"/>
+    </row>
+    <row r="43" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="6"/>
+      <c r="B43" s="14"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="7"/>
+      <c r="E43" s="8"/>
+      <c r="F43" s="8"/>
+    </row>
+    <row r="44" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="6"/>
+      <c r="B44" s="14"/>
+      <c r="C44" s="11"/>
+      <c r="D44" s="7"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="8"/>
+    </row>
+    <row r="45" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="6"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="11"/>
+      <c r="D45" s="7"/>
+      <c r="E45" s="8"/>
+      <c r="F45" s="8"/>
+    </row>
+    <row r="46" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="6"/>
+      <c r="B46" s="14"/>
+      <c r="C46" s="11"/>
+      <c r="D46" s="7"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8"/>
+    </row>
+    <row r="47" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="6"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="11"/>
+      <c r="D47" s="7"/>
+      <c r="E47" s="8"/>
+      <c r="F47" s="8"/>
+    </row>
+    <row r="48" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="6"/>
+      <c r="B48" s="14"/>
+      <c r="C48" s="11"/>
+      <c r="D48" s="7"/>
+      <c r="E48" s="8"/>
+      <c r="F48" s="8"/>
+    </row>
+    <row r="49" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="6"/>
+      <c r="B49" s="14"/>
+      <c r="C49" s="11"/>
+      <c r="D49" s="7"/>
+      <c r="E49" s="8"/>
+      <c r="F49" s="8"/>
+    </row>
+    <row r="50" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="6"/>
+      <c r="B50" s="14"/>
+      <c r="C50" s="11"/>
+      <c r="D50" s="7"/>
+      <c r="E50" s="8"/>
+      <c r="F50" s="8"/>
+    </row>
+    <row r="51" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="6"/>
+      <c r="B51" s="14"/>
+      <c r="C51" s="11"/>
+      <c r="D51" s="7"/>
+      <c r="E51" s="8"/>
+      <c r="F51" s="8"/>
+    </row>
+    <row r="52" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="6"/>
+      <c r="B52" s="14"/>
+      <c r="C52" s="11"/>
+      <c r="D52" s="7"/>
+      <c r="E52" s="8"/>
+      <c r="F52" s="8"/>
+    </row>
+    <row r="53" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="6"/>
+      <c r="B53" s="14"/>
+      <c r="C53" s="11"/>
+      <c r="D53" s="7"/>
+      <c r="E53" s="8"/>
+      <c r="F53" s="8"/>
+    </row>
+    <row r="54" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="6"/>
+      <c r="B54" s="14"/>
+      <c r="C54" s="11"/>
+      <c r="D54" s="7"/>
+      <c r="E54" s="8"/>
+      <c r="F54" s="8"/>
+    </row>
+    <row r="55" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="6"/>
+      <c r="B55" s="14"/>
+      <c r="C55" s="11"/>
+      <c r="D55" s="7"/>
+      <c r="E55" s="8"/>
+      <c r="F55" s="8"/>
+    </row>
+    <row r="56" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="6"/>
+      <c r="B56" s="14"/>
+      <c r="C56" s="11"/>
+      <c r="D56" s="7"/>
+      <c r="E56" s="8"/>
+      <c r="F56" s="8"/>
+    </row>
+    <row r="57" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="6"/>
+      <c r="B57" s="14"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="7"/>
+      <c r="E57" s="8"/>
+      <c r="F57" s="8"/>
+    </row>
+    <row r="58" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="6"/>
+      <c r="B58" s="14"/>
+      <c r="C58" s="11"/>
+      <c r="D58" s="7"/>
+      <c r="E58" s="8"/>
+      <c r="F58" s="8"/>
+    </row>
+    <row r="59" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="6"/>
+      <c r="B59" s="14"/>
+      <c r="C59" s="11"/>
+      <c r="D59" s="7"/>
+      <c r="E59" s="8"/>
+      <c r="F59" s="8"/>
+    </row>
+    <row r="60" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="6"/>
+      <c r="B60" s="14"/>
+      <c r="C60" s="11"/>
+      <c r="D60" s="7"/>
+      <c r="E60" s="8"/>
+      <c r="F60" s="8"/>
+    </row>
+    <row r="61" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="6"/>
+      <c r="B61" s="14"/>
+      <c r="C61" s="11"/>
+      <c r="D61" s="7"/>
+      <c r="E61" s="8"/>
+      <c r="F61" s="8"/>
+    </row>
+    <row r="62" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="6"/>
+      <c r="B62" s="14"/>
+      <c r="C62" s="11"/>
+      <c r="D62" s="7"/>
+      <c r="E62" s="8"/>
+      <c r="F62" s="8"/>
+    </row>
+    <row r="63" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="6"/>
+      <c r="B63" s="14"/>
+      <c r="C63" s="11"/>
+      <c r="D63" s="7"/>
+      <c r="E63" s="8"/>
+      <c r="F63" s="8"/>
+    </row>
+    <row r="64" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="6"/>
+      <c r="B64" s="14"/>
+      <c r="C64" s="11"/>
+      <c r="D64" s="7"/>
+      <c r="E64" s="8"/>
+      <c r="F64" s="8"/>
+    </row>
+    <row r="65" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="6"/>
+      <c r="B65" s="14"/>
+      <c r="C65" s="11"/>
+      <c r="D65" s="7"/>
+      <c r="E65" s="8"/>
+      <c r="F65" s="8"/>
+    </row>
+    <row r="66" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="6"/>
+      <c r="B66" s="14"/>
+      <c r="C66" s="11"/>
+      <c r="D66" s="7"/>
+      <c r="E66" s="8"/>
+      <c r="F66" s="8"/>
+    </row>
+    <row r="67" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="6"/>
+      <c r="B67" s="14"/>
+      <c r="C67" s="11"/>
+      <c r="D67" s="7"/>
+      <c r="E67" s="8"/>
+      <c r="F67" s="8"/>
+    </row>
+    <row r="68" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="6"/>
+      <c r="B68" s="14"/>
+      <c r="C68" s="11"/>
+      <c r="D68" s="7"/>
+      <c r="E68" s="8"/>
+      <c r="F68" s="8"/>
+    </row>
+    <row r="69" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="6"/>
+      <c r="B69" s="14"/>
+      <c r="C69" s="11"/>
+      <c r="D69" s="7"/>
+      <c r="E69" s="8"/>
+      <c r="F69" s="8"/>
+    </row>
+    <row r="70" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="6"/>
+      <c r="B70" s="14"/>
+      <c r="C70" s="11"/>
+      <c r="D70" s="7"/>
+      <c r="E70" s="8"/>
+      <c r="F70" s="8"/>
+    </row>
+    <row r="71" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="6"/>
+      <c r="B71" s="14"/>
+      <c r="C71" s="11"/>
+      <c r="D71" s="7"/>
+      <c r="E71" s="8"/>
+      <c r="F71" s="8"/>
+    </row>
+    <row r="72" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="6"/>
+      <c r="B72" s="14"/>
+      <c r="C72" s="11"/>
+      <c r="D72" s="7"/>
+      <c r="E72" s="8"/>
+      <c r="F72" s="8"/>
+    </row>
+    <row r="73" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="6"/>
+      <c r="B73" s="14"/>
+      <c r="C73" s="11"/>
+      <c r="D73" s="7"/>
+      <c r="E73" s="8"/>
+      <c r="F73" s="8"/>
+    </row>
+    <row r="74" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="6"/>
+      <c r="B74" s="14"/>
+      <c r="C74" s="11"/>
+      <c r="D74" s="7"/>
+      <c r="E74" s="8"/>
+      <c r="F74" s="8"/>
+    </row>
+    <row r="75" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="6"/>
+      <c r="B75" s="14"/>
+      <c r="C75" s="11"/>
+      <c r="D75" s="7"/>
+      <c r="E75" s="8"/>
+      <c r="F75" s="8"/>
+    </row>
+    <row r="76" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="6"/>
+      <c r="B76" s="14"/>
+      <c r="C76" s="11"/>
+      <c r="D76" s="7"/>
+      <c r="E76" s="8"/>
+      <c r="F76" s="8"/>
+    </row>
+    <row r="77" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="6"/>
+      <c r="B77" s="14"/>
+      <c r="C77" s="11"/>
+      <c r="D77" s="7"/>
+      <c r="E77" s="8"/>
+      <c r="F77" s="8"/>
+    </row>
+    <row r="78" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="6"/>
+      <c r="B78" s="14"/>
+      <c r="C78" s="11"/>
+      <c r="D78" s="7"/>
+      <c r="E78" s="8"/>
+      <c r="F78" s="8"/>
+    </row>
+    <row r="79" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="6"/>
+      <c r="B79" s="14"/>
+      <c r="C79" s="11"/>
+      <c r="D79" s="7"/>
+      <c r="E79" s="8"/>
+      <c r="F79" s="8"/>
+    </row>
+    <row r="80" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="6"/>
+      <c r="B80" s="14"/>
+      <c r="C80" s="11"/>
+      <c r="D80" s="7"/>
+      <c r="E80" s="8"/>
+      <c r="F80" s="8"/>
+    </row>
+    <row r="81" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="6"/>
+      <c r="B81" s="14"/>
+      <c r="C81" s="11"/>
+      <c r="D81" s="7"/>
+      <c r="E81" s="8"/>
+      <c r="F81" s="8"/>
+    </row>
+    <row r="82" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="6"/>
+      <c r="B82" s="14"/>
+      <c r="C82" s="11"/>
+      <c r="D82" s="7"/>
+      <c r="E82" s="8"/>
+      <c r="F82" s="8"/>
+    </row>
+    <row r="83" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="6"/>
+      <c r="B83" s="14"/>
+      <c r="C83" s="11"/>
+      <c r="D83" s="7"/>
+      <c r="E83" s="8"/>
+      <c r="F83" s="8"/>
+    </row>
+    <row r="84" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="6"/>
+      <c r="B84" s="14"/>
+      <c r="C84" s="11"/>
+      <c r="D84" s="7"/>
+      <c r="E84" s="8"/>
+      <c r="F84" s="8"/>
+    </row>
+    <row r="85" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="6"/>
+      <c r="B85" s="14"/>
+      <c r="C85" s="11"/>
+      <c r="D85" s="7"/>
+      <c r="E85" s="8"/>
+      <c r="F85" s="8"/>
+    </row>
+    <row r="86" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="6"/>
+      <c r="B86" s="14"/>
+      <c r="C86" s="11"/>
+      <c r="D86" s="7"/>
+      <c r="E86" s="8"/>
+      <c r="F86" s="8"/>
+    </row>
+    <row r="87" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="6"/>
+      <c r="B87" s="14"/>
+      <c r="C87" s="11"/>
+      <c r="D87" s="7"/>
+      <c r="E87" s="8"/>
+      <c r="F87" s="8"/>
+    </row>
+    <row r="88" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="6"/>
+      <c r="B88" s="14"/>
+      <c r="C88" s="11"/>
+      <c r="D88" s="7"/>
+      <c r="E88" s="8"/>
+      <c r="F88" s="8"/>
+    </row>
+    <row r="89" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="6"/>
+      <c r="B89" s="14"/>
+      <c r="C89" s="11"/>
+      <c r="D89" s="7"/>
+      <c r="E89" s="8"/>
+      <c r="F89" s="8"/>
+    </row>
+    <row r="90" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="6"/>
+      <c r="B90" s="14"/>
+      <c r="C90" s="11"/>
+      <c r="D90" s="7"/>
+      <c r="E90" s="8"/>
+      <c r="F90" s="8"/>
+    </row>
+    <row r="91" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="6"/>
+      <c r="B91" s="14"/>
+      <c r="C91" s="11"/>
+      <c r="D91" s="7"/>
+      <c r="E91" s="8"/>
+      <c r="F91" s="8"/>
+    </row>
+    <row r="92" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="6"/>
+      <c r="B92" s="14"/>
+      <c r="C92" s="11"/>
+      <c r="D92" s="7"/>
+      <c r="E92" s="8"/>
+      <c r="F92" s="8"/>
+    </row>
+    <row r="93" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="6"/>
+      <c r="B93" s="14"/>
+      <c r="C93" s="11"/>
+      <c r="D93" s="7"/>
+      <c r="E93" s="8"/>
+      <c r="F93" s="8"/>
+    </row>
+    <row r="94" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="6"/>
+      <c r="B94" s="14"/>
+      <c r="C94" s="11"/>
+      <c r="D94" s="7"/>
+      <c r="E94" s="8"/>
+      <c r="F94" s="8"/>
+    </row>
+    <row r="95" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="6"/>
+      <c r="B95" s="14"/>
+      <c r="C95" s="11"/>
+      <c r="D95" s="7"/>
+      <c r="E95" s="8"/>
+      <c r="F95" s="8"/>
+    </row>
+    <row r="96" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A96" s="6"/>
+      <c r="B96" s="14"/>
+      <c r="C96" s="11"/>
+      <c r="D96" s="7"/>
+      <c r="E96" s="8"/>
+      <c r="F96" s="8"/>
+    </row>
+    <row r="97" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="6"/>
+      <c r="B97" s="14"/>
+      <c r="C97" s="11"/>
+      <c r="D97" s="7"/>
+      <c r="E97" s="8"/>
+      <c r="F97" s="8"/>
+    </row>
+    <row r="98" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="6"/>
+      <c r="B98" s="14"/>
+      <c r="C98" s="11"/>
+      <c r="D98" s="7"/>
+      <c r="E98" s="8"/>
+      <c r="F98" s="8"/>
+    </row>
+    <row r="99" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="6"/>
+      <c r="B99" s="14"/>
+      <c r="C99" s="11"/>
+      <c r="D99" s="7"/>
+      <c r="E99" s="8"/>
+      <c r="F99" s="8"/>
+    </row>
+    <row r="100" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="6"/>
+      <c r="B100" s="14"/>
+      <c r="C100" s="11"/>
+      <c r="D100" s="7"/>
+      <c r="E100" s="8"/>
+      <c r="F100" s="8"/>
+    </row>
+    <row r="101" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A101" s="6"/>
+      <c r="B101" s="14"/>
+      <c r="C101" s="11"/>
+      <c r="D101" s="7"/>
+      <c r="E101" s="8"/>
+      <c r="F101" s="8"/>
+    </row>
+    <row r="102" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="6"/>
+      <c r="B102" s="14"/>
+      <c r="C102" s="11"/>
+      <c r="D102" s="7"/>
+      <c r="E102" s="8"/>
+      <c r="F102" s="8"/>
+    </row>
+    <row r="103" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A103" s="6"/>
+      <c r="B103" s="14"/>
+      <c r="C103" s="11"/>
+      <c r="D103" s="7"/>
+      <c r="E103" s="8"/>
+      <c r="F103" s="8"/>
+    </row>
+    <row r="104" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="6"/>
+      <c r="B104" s="14"/>
+      <c r="C104" s="11"/>
+      <c r="D104" s="7"/>
+      <c r="E104" s="8"/>
+      <c r="F104" s="8"/>
+    </row>
+    <row r="105" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A105" s="6"/>
+      <c r="B105" s="14"/>
+      <c r="C105" s="11"/>
+      <c r="D105" s="7"/>
+      <c r="E105" s="8"/>
+      <c r="F105" s="8"/>
+    </row>
+    <row r="106" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A106" s="6"/>
+      <c r="B106" s="14"/>
+      <c r="C106" s="11"/>
+      <c r="D106" s="7"/>
+      <c r="E106" s="8"/>
+      <c r="F106" s="8"/>
+    </row>
+    <row r="107" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A107" s="6"/>
+      <c r="B107" s="14"/>
+      <c r="C107" s="11"/>
+      <c r="D107" s="7"/>
+      <c r="E107" s="8"/>
+      <c r="F107" s="8"/>
+    </row>
+    <row r="108" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A108" s="6"/>
+      <c r="B108" s="14"/>
+      <c r="C108" s="11"/>
+      <c r="D108" s="7"/>
+      <c r="E108" s="8"/>
+      <c r="F108" s="8"/>
+    </row>
+    <row r="109" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A109" s="6"/>
+      <c r="B109" s="14"/>
+      <c r="C109" s="11"/>
+      <c r="D109" s="7"/>
+      <c r="E109" s="8"/>
+      <c r="F109" s="8"/>
+    </row>
+    <row r="110" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A110" s="6"/>
+      <c r="B110" s="14"/>
+      <c r="C110" s="11"/>
+      <c r="D110" s="7"/>
+      <c r="E110" s="8"/>
+      <c r="F110" s="8"/>
+    </row>
+    <row r="111" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A111" s="6"/>
+      <c r="B111" s="14"/>
+      <c r="C111" s="11"/>
+      <c r="D111" s="7"/>
+      <c r="E111" s="8"/>
+      <c r="F111" s="8"/>
+    </row>
+    <row r="112" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A112" s="6"/>
+      <c r="B112" s="14"/>
+      <c r="C112" s="11"/>
+      <c r="D112" s="7"/>
+      <c r="E112" s="8"/>
+      <c r="F112" s="8"/>
+    </row>
+    <row r="113" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A113" s="6"/>
+      <c r="B113" s="14"/>
+      <c r="C113" s="11"/>
+      <c r="D113" s="7"/>
+      <c r="E113" s="8"/>
+      <c r="F113" s="8"/>
+    </row>
+    <row r="114" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A114" s="6"/>
+      <c r="B114" s="14"/>
+      <c r="C114" s="11"/>
+      <c r="D114" s="7"/>
+      <c r="E114" s="8"/>
+      <c r="F114" s="8"/>
+    </row>
+    <row r="115" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A115" s="6"/>
+      <c r="B115" s="14"/>
+      <c r="C115" s="11"/>
+      <c r="D115" s="7"/>
+      <c r="E115" s="8"/>
+      <c r="F115" s="8"/>
+    </row>
+    <row r="116" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A116" s="6"/>
+      <c r="B116" s="14"/>
+      <c r="C116" s="11"/>
+      <c r="D116" s="7"/>
+      <c r="E116" s="8"/>
+      <c r="F116" s="8"/>
+    </row>
+    <row r="117" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A117" s="6"/>
+      <c r="B117" s="14"/>
+      <c r="C117" s="11"/>
+      <c r="D117" s="7"/>
+      <c r="E117" s="8"/>
+      <c r="F117" s="8"/>
+    </row>
+    <row r="118" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A118" s="6"/>
+      <c r="B118" s="14"/>
+      <c r="C118" s="11"/>
+      <c r="D118" s="7"/>
+      <c r="E118" s="8"/>
+      <c r="F118" s="8"/>
+    </row>
+    <row r="119" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A119" s="6"/>
+      <c r="B119" s="14"/>
+      <c r="C119" s="11"/>
+      <c r="D119" s="7"/>
+      <c r="E119" s="8"/>
+      <c r="F119" s="8"/>
+    </row>
+    <row r="120" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A120" s="6"/>
+      <c r="B120" s="14"/>
+      <c r="C120" s="11"/>
+      <c r="D120" s="7"/>
+      <c r="E120" s="8"/>
+      <c r="F120" s="8"/>
+    </row>
+    <row r="121" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A121" s="6"/>
+      <c r="B121" s="14"/>
+      <c r="C121" s="11"/>
+      <c r="D121" s="7"/>
+      <c r="E121" s="8"/>
+      <c r="F121" s="8"/>
+    </row>
+    <row r="122" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A122" s="6"/>
+      <c r="B122" s="14"/>
+      <c r="C122" s="11"/>
+      <c r="D122" s="7"/>
+      <c r="E122" s="8"/>
+      <c r="F122" s="8"/>
+    </row>
+    <row r="123" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A123" s="6"/>
+      <c r="B123" s="14"/>
+      <c r="C123" s="11"/>
+      <c r="D123" s="7"/>
+      <c r="E123" s="8"/>
+      <c r="F123" s="8"/>
+    </row>
+    <row r="124" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A124" s="6"/>
+      <c r="B124" s="14"/>
+      <c r="C124" s="11"/>
+      <c r="D124" s="7"/>
+      <c r="E124" s="8"/>
+      <c r="F124" s="8"/>
+    </row>
+    <row r="125" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A125" s="6"/>
+      <c r="B125" s="14"/>
+      <c r="C125" s="11"/>
+      <c r="D125" s="7"/>
+      <c r="E125" s="8"/>
+      <c r="F125" s="8"/>
+    </row>
+    <row r="126" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A126" s="6"/>
+      <c r="B126" s="14"/>
+      <c r="C126" s="11"/>
+      <c r="D126" s="7"/>
+      <c r="E126" s="8"/>
+      <c r="F126" s="8"/>
+    </row>
+    <row r="127" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A127" s="6"/>
+      <c r="B127" s="14"/>
+      <c r="C127" s="11"/>
+      <c r="D127" s="7"/>
+      <c r="E127" s="8"/>
+      <c r="F127" s="8"/>
+    </row>
+    <row r="128" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A128" s="6"/>
+      <c r="B128" s="14"/>
+      <c r="C128" s="11"/>
+      <c r="D128" s="7"/>
+      <c r="E128" s="8"/>
+      <c r="F128" s="8"/>
+    </row>
+    <row r="129" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A129" s="6"/>
+      <c r="B129" s="14"/>
+      <c r="C129" s="11"/>
+      <c r="D129" s="7"/>
+      <c r="E129" s="8"/>
+      <c r="F129" s="8"/>
+    </row>
+    <row r="130" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A130" s="6"/>
+      <c r="B130" s="14"/>
+      <c r="C130" s="11"/>
+      <c r="D130" s="7"/>
+      <c r="E130" s="8"/>
+      <c r="F130" s="8"/>
+    </row>
+    <row r="131" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A131" s="6"/>
+      <c r="B131" s="14"/>
+      <c r="C131" s="11"/>
+      <c r="D131" s="7"/>
+      <c r="E131" s="8"/>
+      <c r="F131" s="8"/>
+    </row>
+    <row r="132" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A132" s="6"/>
+      <c r="B132" s="14"/>
+      <c r="C132" s="11"/>
+      <c r="D132" s="7"/>
+      <c r="E132" s="8"/>
+      <c r="F132" s="8"/>
+    </row>
+    <row r="133" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A133" s="6"/>
+      <c r="B133" s="14"/>
+      <c r="C133" s="11"/>
+      <c r="D133" s="7"/>
+      <c r="E133" s="8"/>
+      <c r="F133" s="8"/>
+    </row>
+    <row r="134" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A134" s="6"/>
+      <c r="B134" s="14"/>
+      <c r="C134" s="11"/>
+      <c r="D134" s="7"/>
+      <c r="E134" s="8"/>
+      <c r="F134" s="8"/>
+    </row>
+    <row r="135" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A135" s="6"/>
+      <c r="B135" s="14"/>
+      <c r="C135" s="11"/>
+      <c r="D135" s="7"/>
+      <c r="E135" s="8"/>
+      <c r="F135" s="8"/>
+    </row>
+    <row r="136" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A136" s="6"/>
+      <c r="B136" s="14"/>
+      <c r="C136" s="11"/>
+      <c r="D136" s="7"/>
+      <c r="E136" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F136" s="8"/>
+    </row>
+    <row r="137" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A137" s="6"/>
+      <c r="B137" s="14"/>
+      <c r="C137" s="11"/>
+      <c r="D137" s="7"/>
+      <c r="E137" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F137" s="8"/>
+    </row>
+    <row r="138" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A138" s="6"/>
+      <c r="B138" s="14"/>
+      <c r="C138" s="11"/>
+      <c r="D138" s="7"/>
+      <c r="E138" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="F32" s="8"/>
-    </row>
-    <row r="33" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="6">
-        <v>46044</v>
-      </c>
-      <c r="B33" s="14">
-        <v>2</v>
-      </c>
-      <c r="C33" s="11">
-        <v>0.75</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F33" s="8"/>
-    </row>
-    <row r="34" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="6">
-        <v>46045</v>
-      </c>
-      <c r="B34" s="14">
-        <v>2</v>
-      </c>
-      <c r="C34" s="11">
-        <v>2</v>
-      </c>
-      <c r="D34" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E34" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="F34" s="8"/>
-    </row>
-    <row r="35" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="6">
-        <v>46046</v>
-      </c>
-      <c r="B35" s="14">
-        <v>2</v>
-      </c>
-      <c r="C35" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D35" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E35" s="8" t="s">
+      <c r="F138" s="8"/>
+    </row>
+    <row r="139" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A139" s="6"/>
+      <c r="B139" s="14"/>
+      <c r="C139" s="11"/>
+      <c r="D139" s="7"/>
+      <c r="E139" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F35" s="8"/>
-    </row>
-    <row r="36" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="6">
-        <v>46047</v>
-      </c>
-      <c r="B36" s="14">
-        <v>2</v>
-      </c>
-      <c r="C36" s="11">
-        <v>1</v>
-      </c>
-      <c r="D36" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E36" s="8" t="s">
+      <c r="F139" s="8"/>
+    </row>
+    <row r="140" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A140" s="6"/>
+      <c r="B140" s="14"/>
+      <c r="C140" s="11"/>
+      <c r="D140" s="7"/>
+      <c r="E140" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="F36" s="8"/>
-    </row>
-    <row r="37" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="6">
-        <v>46048</v>
-      </c>
-      <c r="B37" s="14">
-        <v>2</v>
-      </c>
-      <c r="C37" s="11">
-        <v>1.75</v>
-      </c>
-      <c r="D37" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E37" s="8" t="s">
+      <c r="F140" s="8"/>
+    </row>
+    <row r="141" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A141" s="6"/>
+      <c r="B141" s="14"/>
+      <c r="C141" s="11"/>
+      <c r="D141" s="7"/>
+      <c r="E141" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="F37" s="8"/>
-    </row>
-    <row r="38" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="6">
-        <v>46049</v>
-      </c>
-      <c r="B38" s="14">
-        <v>2</v>
-      </c>
-      <c r="C38" s="11">
-        <v>0.25</v>
-      </c>
-      <c r="D38" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E38" s="8" t="s">
+      <c r="F141" s="8"/>
+    </row>
+    <row r="142" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A142" s="6"/>
+      <c r="B142" s="14"/>
+      <c r="C142" s="11"/>
+      <c r="D142" s="7"/>
+      <c r="E142" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="F38" s="8"/>
-    </row>
-    <row r="39" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="6">
-        <v>46050</v>
-      </c>
-      <c r="B39" s="14">
-        <v>2</v>
-      </c>
-      <c r="C39" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D39" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E39" s="8" t="s">
+      <c r="F142" s="8"/>
+    </row>
+    <row r="143" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A143" s="6"/>
+      <c r="B143" s="14"/>
+      <c r="C143" s="11"/>
+      <c r="D143" s="7"/>
+      <c r="E143" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="F39" s="8"/>
-    </row>
-    <row r="40" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="6">
-        <v>46051</v>
-      </c>
-      <c r="B40" s="14">
-        <v>2</v>
-      </c>
-      <c r="C40" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="D40" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E40" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="F40" s="8"/>
-    </row>
-    <row r="41" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="6">
-        <v>46052</v>
-      </c>
-      <c r="B41" s="14">
-        <v>2</v>
-      </c>
-      <c r="C41" s="11">
-        <v>1.25</v>
-      </c>
-      <c r="D41" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E41" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="F41" s="8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="6">
-        <v>46053</v>
-      </c>
-      <c r="B42" s="14">
-        <v>2</v>
-      </c>
-      <c r="C42" s="11">
-        <v>2.25</v>
-      </c>
-      <c r="D42" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E42" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="F42" s="8"/>
-    </row>
-    <row r="43" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="6">
-        <v>46054</v>
-      </c>
-      <c r="B43" s="14">
-        <v>2</v>
-      </c>
-      <c r="C43" s="11">
-        <v>1.25</v>
-      </c>
-      <c r="D43" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E43" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="F43" s="8"/>
-    </row>
-    <row r="44" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="6">
-        <v>46055</v>
-      </c>
-      <c r="B44" s="14">
-        <v>2</v>
-      </c>
-      <c r="C44" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D44" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E44" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="F44" s="8"/>
-    </row>
-    <row r="45" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="6">
-        <v>46056</v>
-      </c>
-      <c r="B45" s="14">
-        <v>2</v>
-      </c>
-      <c r="C45" s="11">
-        <v>0.75</v>
-      </c>
-      <c r="D45" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E45" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="F45" s="8"/>
-    </row>
-    <row r="46" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="6">
-        <v>46057</v>
-      </c>
-      <c r="B46" s="14">
-        <v>2</v>
-      </c>
-      <c r="C46" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D46" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E46" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F46" s="8"/>
-    </row>
-    <row r="47" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="6">
-        <v>46058</v>
-      </c>
-      <c r="B47" s="14">
-        <v>2</v>
-      </c>
-      <c r="C47" s="11">
-        <v>1.75</v>
-      </c>
-      <c r="D47" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E47" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="F47" s="8"/>
-    </row>
-    <row r="48" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="6">
-        <v>46059</v>
-      </c>
-      <c r="B48" s="14">
-        <v>2</v>
-      </c>
-      <c r="C48" s="11">
-        <v>1</v>
-      </c>
-      <c r="D48" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E48" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="F48" s="8"/>
-    </row>
-    <row r="49" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="6">
-        <v>46060</v>
-      </c>
-      <c r="B49" s="14">
-        <v>2</v>
-      </c>
-      <c r="C49" s="11">
-        <v>1.25</v>
-      </c>
-      <c r="D49" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E49" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="F49" s="8"/>
-    </row>
-    <row r="50" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="6">
-        <v>46061</v>
-      </c>
-      <c r="B50" s="14">
-        <v>2</v>
-      </c>
-      <c r="C50" s="11">
-        <v>0.75</v>
-      </c>
-      <c r="D50" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E50" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="F50" s="8"/>
-    </row>
-    <row r="51" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="6">
-        <v>46062</v>
-      </c>
-      <c r="B51" s="14">
-        <v>2</v>
-      </c>
-      <c r="C51" s="11">
-        <v>0.5</v>
-      </c>
-      <c r="D51" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E51" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="F51" s="8"/>
-    </row>
-    <row r="52" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="6">
-        <v>46063</v>
-      </c>
-      <c r="B52" s="14">
-        <v>2</v>
-      </c>
-      <c r="C52" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="D52" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E52" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="F52" s="8"/>
-    </row>
-    <row r="53" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="6">
-        <v>45057</v>
-      </c>
-      <c r="B53" s="14">
-        <v>2</v>
-      </c>
-      <c r="C53" s="11">
-        <v>0.5</v>
-      </c>
-      <c r="D53" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E53" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="F53" s="8"/>
-    </row>
-    <row r="54" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="6">
-        <v>45057</v>
-      </c>
-      <c r="B54" s="14">
-        <v>2</v>
-      </c>
-      <c r="C54" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="D54" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E54" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="F54" s="8" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="6">
-        <v>45057</v>
-      </c>
-      <c r="B55" s="14">
-        <v>2</v>
-      </c>
-      <c r="C55" s="11">
-        <v>0.25</v>
-      </c>
-      <c r="D55" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E55" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="F55" s="8"/>
-    </row>
-    <row r="56" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="6">
-        <v>45057</v>
-      </c>
-      <c r="B56" s="14">
-        <v>2</v>
-      </c>
-      <c r="C56" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="D56" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E56" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="F56" s="8"/>
-    </row>
-    <row r="57" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="6">
-        <v>45057</v>
-      </c>
-      <c r="B57" s="14">
-        <v>2</v>
-      </c>
-      <c r="C57" s="11">
-        <v>2.25</v>
-      </c>
-      <c r="D57" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E57" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="F57" s="8"/>
-    </row>
-    <row r="58" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="6">
-        <v>45057</v>
-      </c>
-      <c r="B58" s="14">
-        <v>2</v>
-      </c>
-      <c r="C58" s="11">
-        <v>0.5</v>
-      </c>
-      <c r="D58" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E58" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F58" s="8"/>
-    </row>
-    <row r="59" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="6">
-        <v>45057</v>
-      </c>
-      <c r="B59" s="14">
-        <v>2</v>
-      </c>
-      <c r="C59" s="11">
-        <v>0.75</v>
-      </c>
-      <c r="D59" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E59" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="F59" s="8"/>
-    </row>
-    <row r="60" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="6">
-        <v>45057</v>
-      </c>
-      <c r="B60" s="14">
-        <v>2</v>
-      </c>
-      <c r="C60" s="11">
-        <v>2.25</v>
-      </c>
-      <c r="D60" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E60" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="F60" s="8"/>
-    </row>
-    <row r="61" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="6">
-        <v>45057</v>
-      </c>
-      <c r="B61" s="14">
-        <v>2</v>
-      </c>
-      <c r="C61" s="11">
-        <v>1.75</v>
-      </c>
-      <c r="D61" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E61" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F61" s="8" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="6">
-        <v>45057</v>
-      </c>
-      <c r="B62" s="14">
-        <v>2</v>
-      </c>
-      <c r="C62" s="11">
-        <v>2.25</v>
-      </c>
-      <c r="D62" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E62" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="F62" s="8"/>
-    </row>
-    <row r="63" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="6">
-        <v>45058</v>
-      </c>
-      <c r="B63" s="14">
-        <v>2</v>
-      </c>
-      <c r="C63" s="11">
-        <v>0.25</v>
-      </c>
-      <c r="D63" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E63" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="F63" s="8"/>
-    </row>
-    <row r="64" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="6">
-        <v>45058</v>
-      </c>
-      <c r="B64" s="14">
-        <v>2</v>
-      </c>
-      <c r="C64" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D64" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E64" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="F64" s="8" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="6">
-        <v>45058</v>
-      </c>
-      <c r="B65" s="14">
-        <v>2</v>
-      </c>
-      <c r="C65" s="11">
-        <v>1.75</v>
-      </c>
-      <c r="D65" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E65" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="F65" s="8"/>
-    </row>
-    <row r="66" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="6">
-        <v>45058</v>
-      </c>
-      <c r="B66" s="14">
-        <v>2</v>
-      </c>
-      <c r="C66" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="D66" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E66" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F66" s="8"/>
-    </row>
-    <row r="67" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="6">
-        <v>45058</v>
-      </c>
-      <c r="B67" s="14">
-        <v>2</v>
-      </c>
-      <c r="C67" s="11">
-        <v>2</v>
-      </c>
-      <c r="D67" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E67" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="F67" s="8"/>
-    </row>
-    <row r="68" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="6">
-        <v>45058</v>
-      </c>
-      <c r="B68" s="14">
-        <v>2</v>
-      </c>
-      <c r="C68" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="D68" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E68" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F68" s="8" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="6">
-        <v>45058</v>
-      </c>
-      <c r="B69" s="14">
-        <v>2</v>
-      </c>
-      <c r="C69" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D69" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E69" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="F69" s="8"/>
-    </row>
-    <row r="70" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="6">
-        <v>45058</v>
-      </c>
-      <c r="B70" s="14">
-        <v>2</v>
-      </c>
-      <c r="C70" s="11">
-        <v>0.75</v>
-      </c>
-      <c r="D70" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E70" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="F70" s="8"/>
-    </row>
-    <row r="71" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="6">
-        <v>45061</v>
-      </c>
-      <c r="B71" s="14">
-        <v>3</v>
-      </c>
-      <c r="C71" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D71" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E71" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="F71" s="8" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="6">
-        <v>45061</v>
-      </c>
-      <c r="B72" s="14">
-        <v>3</v>
-      </c>
-      <c r="C72" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D72" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E72" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F72" s="8" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="6">
-        <v>45061</v>
-      </c>
-      <c r="B73" s="14">
-        <v>3</v>
-      </c>
-      <c r="C73" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="D73" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E73" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="F73" s="8"/>
-    </row>
-    <row r="74" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="6">
-        <v>45061</v>
-      </c>
-      <c r="B74" s="14">
-        <v>3</v>
-      </c>
-      <c r="C74" s="11">
-        <v>1.75</v>
-      </c>
-      <c r="D74" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E74" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="F74" s="8" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="6">
-        <v>45061</v>
-      </c>
-      <c r="B75" s="14">
-        <v>3</v>
-      </c>
-      <c r="C75" s="11">
-        <v>1.75</v>
-      </c>
-      <c r="D75" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E75" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="F75" s="8"/>
-    </row>
-    <row r="76" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="6">
-        <v>45061</v>
-      </c>
-      <c r="B76" s="14">
-        <v>3</v>
-      </c>
-      <c r="C76" s="11">
-        <v>2.25</v>
-      </c>
-      <c r="D76" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E76" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="F76" s="8"/>
-    </row>
-    <row r="77" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="6">
-        <v>45061</v>
-      </c>
-      <c r="B77" s="14">
-        <v>3</v>
-      </c>
-      <c r="C77" s="11">
-        <v>1</v>
-      </c>
-      <c r="D77" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E77" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="F77" s="8" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="6">
-        <v>45061</v>
-      </c>
-      <c r="B78" s="14">
-        <v>3</v>
-      </c>
-      <c r="C78" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D78" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E78" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="F78" s="8"/>
-    </row>
-    <row r="79" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="6">
-        <v>45062</v>
-      </c>
-      <c r="B79" s="14">
-        <v>3</v>
-      </c>
-      <c r="C79" s="11">
-        <v>1.75</v>
-      </c>
-      <c r="D79" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E79" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="F79" s="8" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="6">
-        <v>45062</v>
-      </c>
-      <c r="B80" s="14">
-        <v>3</v>
-      </c>
-      <c r="C80" s="11">
-        <v>0.75</v>
-      </c>
-      <c r="D80" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E80" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="F80" s="8" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="6">
-        <v>45062</v>
-      </c>
-      <c r="B81" s="14">
-        <v>3</v>
-      </c>
-      <c r="C81" s="11">
-        <v>0.25</v>
-      </c>
-      <c r="D81" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E81" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="F81" s="8"/>
-    </row>
-    <row r="82" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="6">
-        <v>45062</v>
-      </c>
-      <c r="B82" s="14">
-        <v>3</v>
-      </c>
-      <c r="C82" s="11">
-        <v>0.75</v>
-      </c>
-      <c r="D82" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E82" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="F82" s="8" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="6">
-        <v>45062</v>
-      </c>
-      <c r="B83" s="14">
-        <v>3</v>
-      </c>
-      <c r="C83" s="11">
-        <v>1.75</v>
-      </c>
-      <c r="D83" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E83" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="F83" s="8"/>
-    </row>
-    <row r="84" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="6">
-        <v>45062</v>
-      </c>
-      <c r="B84" s="14">
-        <v>3</v>
-      </c>
-      <c r="C84" s="11">
-        <v>1.25</v>
-      </c>
-      <c r="D84" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E84" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="F84" s="8"/>
-    </row>
-    <row r="85" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="6">
-        <v>45062</v>
-      </c>
-      <c r="B85" s="14">
-        <v>3</v>
-      </c>
-      <c r="C85" s="11">
-        <v>1.25</v>
-      </c>
-      <c r="D85" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E85" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="F85" s="8"/>
-    </row>
-    <row r="86" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="6">
-        <v>45062</v>
-      </c>
-      <c r="B86" s="14">
-        <v>3</v>
-      </c>
-      <c r="C86" s="11">
-        <v>0.75</v>
-      </c>
-      <c r="D86" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E86" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="F86" s="8"/>
-    </row>
-    <row r="87" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="6">
-        <v>45062</v>
-      </c>
-      <c r="B87" s="14">
-        <v>3</v>
-      </c>
-      <c r="C87" s="11">
-        <v>0.5</v>
-      </c>
-      <c r="D87" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E87" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="F87" s="8"/>
-    </row>
-    <row r="88" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="6">
-        <v>45062</v>
-      </c>
-      <c r="B88" s="14">
-        <v>3</v>
-      </c>
-      <c r="C88" s="11">
-        <v>0.5</v>
-      </c>
-      <c r="D88" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E88" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="F88" s="8" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A89" s="6">
-        <v>45062</v>
-      </c>
-      <c r="B89" s="14">
-        <v>3</v>
-      </c>
-      <c r="C89" s="11">
-        <v>0.75</v>
-      </c>
-      <c r="D89" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E89" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="F89" s="8"/>
-    </row>
-    <row r="90" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="6">
-        <v>45062</v>
-      </c>
-      <c r="B90" s="14">
-        <v>3</v>
-      </c>
-      <c r="C90" s="11">
-        <v>1</v>
-      </c>
-      <c r="D90" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E90" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="F90" s="8"/>
-    </row>
-    <row r="91" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="6">
-        <v>45062</v>
-      </c>
-      <c r="B91" s="14">
-        <v>3</v>
-      </c>
-      <c r="C91" s="11">
-        <v>2.25</v>
-      </c>
-      <c r="D91" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E91" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="F91" s="8"/>
-    </row>
-    <row r="92" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="6">
-        <v>45062</v>
-      </c>
-      <c r="B92" s="14">
-        <v>3</v>
-      </c>
-      <c r="C92" s="11">
-        <v>2.25</v>
-      </c>
-      <c r="D92" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E92" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="F92" s="8"/>
-    </row>
-    <row r="93" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A93" s="6">
-        <v>45068</v>
-      </c>
-      <c r="B93" s="14">
-        <v>4</v>
-      </c>
-      <c r="C93" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D93" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E93" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="F93" s="8"/>
-    </row>
-    <row r="94" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A94" s="6">
-        <v>45068</v>
-      </c>
-      <c r="B94" s="14">
-        <v>4</v>
-      </c>
-      <c r="C94" s="11">
-        <v>0.75</v>
-      </c>
-      <c r="D94" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E94" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="F94" s="8" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A95" s="6">
-        <v>45068</v>
-      </c>
-      <c r="B95" s="14">
-        <v>4</v>
-      </c>
-      <c r="C95" s="11">
-        <v>1</v>
-      </c>
-      <c r="D95" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E95" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="F95" s="8"/>
-    </row>
-    <row r="96" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="6">
-        <v>45068</v>
-      </c>
-      <c r="B96" s="14">
-        <v>4</v>
-      </c>
-      <c r="C96" s="11">
-        <v>1.25</v>
-      </c>
-      <c r="D96" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E96" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="F96" s="8" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="6">
-        <v>45068</v>
-      </c>
-      <c r="B97" s="14">
-        <v>4</v>
-      </c>
-      <c r="C97" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D97" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E97" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="F97" s="8"/>
-    </row>
-    <row r="98" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="6">
-        <v>45068</v>
-      </c>
-      <c r="B98" s="14">
-        <v>4</v>
-      </c>
-      <c r="C98" s="11">
-        <v>1</v>
-      </c>
-      <c r="D98" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E98" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F98" s="8" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="6">
-        <v>45068</v>
-      </c>
-      <c r="B99" s="14">
-        <v>4</v>
-      </c>
-      <c r="C99" s="11">
-        <v>2.25</v>
-      </c>
-      <c r="D99" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E99" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="F99" s="8"/>
-    </row>
-    <row r="100" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A100" s="6">
-        <v>45068</v>
-      </c>
-      <c r="B100" s="14">
-        <v>4</v>
-      </c>
-      <c r="C100" s="11">
-        <v>1.75</v>
-      </c>
-      <c r="D100" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E100" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="F100" s="8"/>
-    </row>
-    <row r="101" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A101" s="6">
-        <v>45068</v>
-      </c>
-      <c r="B101" s="14">
-        <v>4</v>
-      </c>
-      <c r="C101" s="11">
-        <v>1.25</v>
-      </c>
-      <c r="D101" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E101" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="F101" s="8"/>
-    </row>
-    <row r="102" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A102" s="6">
-        <v>45068</v>
-      </c>
-      <c r="B102" s="14">
-        <v>4</v>
-      </c>
-      <c r="C102" s="11">
-        <v>0.25</v>
-      </c>
-      <c r="D102" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E102" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="F102" s="8"/>
-    </row>
-    <row r="103" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A103" s="6">
-        <v>45068</v>
-      </c>
-      <c r="B103" s="14">
-        <v>4</v>
-      </c>
-      <c r="C103" s="11">
-        <v>0.75</v>
-      </c>
-      <c r="D103" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E103" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="F103" s="8"/>
-    </row>
-    <row r="104" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A104" s="6">
-        <v>45068</v>
-      </c>
-      <c r="B104" s="14">
-        <v>4</v>
-      </c>
-      <c r="C104" s="11">
-        <v>1.25</v>
-      </c>
-      <c r="D104" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E104" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="F104" s="8"/>
-    </row>
-    <row r="105" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A105" s="6">
-        <v>45068</v>
-      </c>
-      <c r="B105" s="14">
-        <v>4</v>
-      </c>
-      <c r="C105" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="D105" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E105" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="F105" s="8"/>
-    </row>
-    <row r="106" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A106" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B106" s="14">
-        <v>4</v>
-      </c>
-      <c r="C106" s="11">
-        <v>2.25</v>
-      </c>
-      <c r="D106" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E106" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="F106" s="8"/>
-    </row>
-    <row r="107" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A107" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B107" s="14">
-        <v>4</v>
-      </c>
-      <c r="C107" s="11">
-        <v>1.25</v>
-      </c>
-      <c r="D107" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E107" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="F107" s="8"/>
-    </row>
-    <row r="108" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A108" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B108" s="14">
-        <v>4</v>
-      </c>
-      <c r="C108" s="11">
-        <v>0.5</v>
-      </c>
-      <c r="D108" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E108" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="F108" s="8"/>
-    </row>
-    <row r="109" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A109" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B109" s="14">
-        <v>4</v>
-      </c>
-      <c r="C109" s="11">
-        <v>1.25</v>
-      </c>
-      <c r="D109" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E109" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="F109" s="8" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B110" s="14">
-        <v>4</v>
-      </c>
-      <c r="C110" s="11">
-        <v>2</v>
-      </c>
-      <c r="D110" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E110" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="F110" s="8" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A111" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B111" s="14">
-        <v>4</v>
-      </c>
-      <c r="C111" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="D111" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E111" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="F111" s="8"/>
-    </row>
-    <row r="112" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A112" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B112" s="14">
-        <v>4</v>
-      </c>
-      <c r="C112" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D112" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E112" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="F112" s="8"/>
-    </row>
-    <row r="113" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A113" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B113" s="14">
-        <v>4</v>
-      </c>
-      <c r="C113" s="11">
-        <v>2.25</v>
-      </c>
-      <c r="D113" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E113" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="F113" s="8"/>
-    </row>
-    <row r="114" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A114" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B114" s="14">
-        <v>4</v>
-      </c>
-      <c r="C114" s="11">
-        <v>0.5</v>
-      </c>
-      <c r="D114" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E114" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F114" s="8"/>
-    </row>
-    <row r="115" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A115" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B115" s="14">
-        <v>4</v>
-      </c>
-      <c r="C115" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D115" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E115" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="F115" s="8" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A116" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B116" s="14">
-        <v>4</v>
-      </c>
-      <c r="C116" s="11">
-        <v>1.25</v>
-      </c>
-      <c r="D116" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E116" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="F116" s="8"/>
-    </row>
-    <row r="117" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A117" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B117" s="14">
-        <v>4</v>
-      </c>
-      <c r="C117" s="11">
-        <v>2.25</v>
-      </c>
-      <c r="D117" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E117" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="F117" s="8"/>
-    </row>
-    <row r="118" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A118" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B118" s="14">
-        <v>4</v>
-      </c>
-      <c r="C118" s="11">
-        <v>0.25</v>
-      </c>
-      <c r="D118" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E118" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="F118" s="8"/>
-    </row>
-    <row r="119" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A119" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B119" s="14">
-        <v>4</v>
-      </c>
-      <c r="C119" s="11">
-        <v>2.25</v>
-      </c>
-      <c r="D119" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E119" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="F119" s="8"/>
-    </row>
-    <row r="120" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A120" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B120" s="14">
-        <v>4</v>
-      </c>
-      <c r="C120" s="11">
-        <v>1</v>
-      </c>
-      <c r="D120" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E120" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="F120" s="8"/>
-    </row>
-    <row r="121" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A121" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B121" s="14">
-        <v>4</v>
-      </c>
-      <c r="C121" s="11">
-        <v>2</v>
-      </c>
-      <c r="D121" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E121" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="F121" s="8"/>
-    </row>
-    <row r="122" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A122" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B122" s="14">
-        <v>4</v>
-      </c>
-      <c r="C122" s="11">
-        <v>2</v>
-      </c>
-      <c r="D122" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E122" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="F122" s="8"/>
-    </row>
-    <row r="123" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A123" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B123" s="14">
-        <v>4</v>
-      </c>
-      <c r="C123" s="11">
-        <v>1.75</v>
-      </c>
-      <c r="D123" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E123" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="F123" s="8"/>
-    </row>
-    <row r="124" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A124" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B124" s="14">
-        <v>4</v>
-      </c>
-      <c r="C124" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D124" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E124" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="F124" s="8"/>
-    </row>
-    <row r="125" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A125" s="6">
-        <v>45069</v>
-      </c>
-      <c r="B125" s="14">
-        <v>4</v>
-      </c>
-      <c r="C125" s="11">
-        <v>1.75</v>
-      </c>
-      <c r="D125" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E125" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="F125" s="8"/>
-    </row>
-    <row r="126" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="6">
-        <v>45071</v>
-      </c>
-      <c r="B126" s="14">
-        <v>4</v>
-      </c>
-      <c r="C126" s="11">
-        <v>0.75</v>
-      </c>
-      <c r="D126" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E126" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="F126" s="8" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="127" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A127" s="6">
-        <v>45071</v>
-      </c>
-      <c r="B127" s="14">
-        <v>4</v>
-      </c>
-      <c r="C127" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D127" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E127" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="F127" s="8"/>
-    </row>
-    <row r="128" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A128" s="6">
-        <v>45071</v>
-      </c>
-      <c r="B128" s="14">
-        <v>4</v>
-      </c>
-      <c r="C128" s="11">
-        <v>0.25</v>
-      </c>
-      <c r="D128" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E128" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="F128" s="8"/>
-    </row>
-    <row r="129" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A129" s="6">
-        <v>45071</v>
-      </c>
-      <c r="B129" s="14">
-        <v>4</v>
-      </c>
-      <c r="C129" s="11">
-        <v>0.5</v>
-      </c>
-      <c r="D129" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E129" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="F129" s="8"/>
-    </row>
-    <row r="130" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A130" s="6">
-        <v>45071</v>
-      </c>
-      <c r="B130" s="14">
-        <v>4</v>
-      </c>
-      <c r="C130" s="11">
-        <v>1.75</v>
-      </c>
-      <c r="D130" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E130" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="F130" s="8"/>
-    </row>
-    <row r="131" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A131" s="6">
-        <v>45071</v>
-      </c>
-      <c r="B131" s="14">
-        <v>4</v>
-      </c>
-      <c r="C131" s="11">
-        <v>1</v>
-      </c>
-      <c r="D131" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E131" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="F131" s="8"/>
-    </row>
-    <row r="132" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A132" s="6">
-        <v>45071</v>
-      </c>
-      <c r="B132" s="14">
-        <v>4</v>
-      </c>
-      <c r="C132" s="11">
-        <v>1.75</v>
-      </c>
-      <c r="D132" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E132" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="F132" s="8"/>
-    </row>
-    <row r="133" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A133" s="6">
-        <v>45071</v>
-      </c>
-      <c r="B133" s="14">
-        <v>4</v>
-      </c>
-      <c r="C133" s="11">
-        <v>0.75</v>
-      </c>
-      <c r="D133" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E133" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="F133" s="8"/>
-    </row>
-    <row r="134" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A134" s="6">
-        <v>45072</v>
-      </c>
-      <c r="B134" s="14">
-        <v>4</v>
-      </c>
-      <c r="C134" s="11">
-        <v>0.75</v>
-      </c>
-      <c r="D134" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E134" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="F134" s="8" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="135" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A135" s="6">
-        <v>45072</v>
-      </c>
-      <c r="B135" s="14">
-        <v>4</v>
-      </c>
-      <c r="C135" s="11">
-        <v>0.5</v>
-      </c>
-      <c r="D135" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E135" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="F135" s="8" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="136" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A136" s="6">
-        <v>45072</v>
-      </c>
-      <c r="B136" s="14">
-        <v>4</v>
-      </c>
-      <c r="C136" s="11">
-        <v>0.5</v>
-      </c>
-      <c r="D136" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E136" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="F136" s="8"/>
-    </row>
-    <row r="137" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A137" s="6">
-        <v>45072</v>
-      </c>
-      <c r="B137" s="14">
-        <v>4</v>
-      </c>
-      <c r="C137" s="11">
-        <v>0.5</v>
-      </c>
-      <c r="D137" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E137" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="F137" s="8"/>
-    </row>
-    <row r="138" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A138" s="6">
-        <v>45076</v>
-      </c>
-      <c r="B138" s="14">
-        <v>5</v>
-      </c>
-      <c r="C138" s="11">
-        <v>1.25</v>
-      </c>
-      <c r="D138" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E138" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="F138" s="8"/>
-    </row>
-    <row r="139" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A139" s="6">
-        <v>45076</v>
-      </c>
-      <c r="B139" s="14">
-        <v>5</v>
-      </c>
-      <c r="C139" s="11">
-        <v>2</v>
-      </c>
-      <c r="D139" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E139" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="F139" s="8"/>
-    </row>
-    <row r="140" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A140" s="6">
-        <v>45076</v>
-      </c>
-      <c r="B140" s="14">
-        <v>5</v>
-      </c>
-      <c r="C140" s="11">
-        <v>2.25</v>
-      </c>
-      <c r="D140" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E140" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="F140" s="8"/>
-    </row>
-    <row r="141" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A141" s="6">
-        <v>45076</v>
-      </c>
-      <c r="B141" s="14">
-        <v>5</v>
-      </c>
-      <c r="C141" s="11">
-        <v>2.25</v>
-      </c>
-      <c r="D141" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E141" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="F141" s="8"/>
-    </row>
-    <row r="142" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A142" s="6">
-        <v>45076</v>
-      </c>
-      <c r="B142" s="14">
-        <v>5</v>
-      </c>
-      <c r="C142" s="11">
-        <v>0.5</v>
-      </c>
-      <c r="D142" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E142" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="F142" s="8"/>
-    </row>
-    <row r="143" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A143" s="6">
-        <v>45076</v>
-      </c>
-      <c r="B143" s="14">
-        <v>5</v>
-      </c>
-      <c r="C143" s="11">
-        <v>1.75</v>
-      </c>
-      <c r="D143" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E143" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="F143" s="8"/>
     </row>
     <row r="144" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A144" s="6">
-        <v>45076</v>
-      </c>
-      <c r="B144" s="14">
-        <v>5</v>
-      </c>
-      <c r="C144" s="11">
-        <v>1.75</v>
-      </c>
-      <c r="D144" s="7" t="s">
-        <v>6</v>
-      </c>
+      <c r="A144" s="6"/>
+      <c r="B144" s="14"/>
+      <c r="C144" s="11"/>
+      <c r="D144" s="7"/>
       <c r="E144" s="8" t="s">
         <v>16</v>
       </c>
       <c r="F144" s="8"/>
     </row>
     <row r="145" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A145" s="6">
-        <v>45076</v>
-      </c>
-      <c r="B145" s="14">
-        <v>5</v>
-      </c>
-      <c r="C145" s="11">
-        <v>2.25</v>
-      </c>
-      <c r="D145" s="7" t="s">
-        <v>11</v>
-      </c>
+      <c r="A145" s="6"/>
+      <c r="B145" s="14"/>
+      <c r="C145" s="11"/>
+      <c r="D145" s="7"/>
       <c r="E145" s="8" t="s">
-        <v>138</v>
+        <v>25</v>
       </c>
       <c r="F145" s="8"/>
     </row>
     <row r="146" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A146" s="6">
-        <v>45076</v>
-      </c>
-      <c r="B146" s="14">
-        <v>5</v>
-      </c>
-      <c r="C146" s="11">
-        <v>1.75</v>
-      </c>
-      <c r="D146" s="7" t="s">
-        <v>11</v>
-      </c>
+      <c r="A146" s="6"/>
+      <c r="B146" s="14"/>
+      <c r="C146" s="11"/>
+      <c r="D146" s="7"/>
       <c r="E146" s="8" t="s">
-        <v>139</v>
+        <v>26</v>
       </c>
       <c r="F146" s="8"/>
     </row>
     <row r="147" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="6">
-        <v>45076</v>
-      </c>
-      <c r="B147" s="14">
-        <v>5</v>
-      </c>
-      <c r="C147" s="11">
-        <v>2</v>
-      </c>
-      <c r="D147" s="7" t="s">
-        <v>11</v>
-      </c>
+      <c r="A147" s="6"/>
+      <c r="B147" s="14"/>
+      <c r="C147" s="11"/>
+      <c r="D147" s="7"/>
       <c r="E147" s="8" t="s">
-        <v>140</v>
+        <v>27</v>
       </c>
       <c r="F147" s="8"/>
     </row>
     <row r="148" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A148" s="6">
-        <v>45076</v>
-      </c>
-      <c r="B148" s="14">
-        <v>5</v>
-      </c>
-      <c r="C148" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D148" s="7" t="s">
-        <v>6</v>
-      </c>
+      <c r="A148" s="6"/>
+      <c r="B148" s="14"/>
+      <c r="C148" s="11"/>
+      <c r="D148" s="7"/>
       <c r="E148" s="8" t="s">
-        <v>128</v>
+        <v>18</v>
       </c>
       <c r="F148" s="8"/>
     </row>
     <row r="149" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A149" s="6">
-        <v>45076</v>
-      </c>
-      <c r="B149" s="14">
-        <v>5</v>
-      </c>
-      <c r="C149" s="11">
-        <v>2</v>
-      </c>
-      <c r="D149" s="7" t="s">
-        <v>6</v>
-      </c>
+      <c r="A149" s="6"/>
+      <c r="B149" s="14"/>
+      <c r="C149" s="11"/>
+      <c r="D149" s="7"/>
       <c r="E149" s="8" t="s">
-        <v>132</v>
+        <v>19</v>
       </c>
       <c r="F149" s="8"/>
     </row>
     <row r="150" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A150" s="6">
-        <v>45078</v>
-      </c>
-      <c r="B150" s="14">
-        <v>5</v>
-      </c>
-      <c r="C150" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D150" s="7" t="s">
-        <v>11</v>
-      </c>
+      <c r="A150" s="6"/>
+      <c r="B150" s="14"/>
+      <c r="C150" s="11"/>
+      <c r="D150" s="7"/>
       <c r="E150" s="8" t="s">
-        <v>141</v>
+        <v>28</v>
       </c>
       <c r="F150" s="8"/>
     </row>
     <row r="151" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A151" s="6">
-        <v>45078</v>
-      </c>
-      <c r="B151" s="14">
-        <v>5</v>
-      </c>
-      <c r="C151" s="11">
-        <v>1.25</v>
-      </c>
-      <c r="D151" s="7" t="s">
-        <v>11</v>
-      </c>
+      <c r="A151" s="6"/>
+      <c r="B151" s="14"/>
+      <c r="C151" s="11"/>
+      <c r="D151" s="7"/>
       <c r="E151" s="8" t="s">
-        <v>142</v>
+        <v>29</v>
       </c>
       <c r="F151" s="8"/>
     </row>
     <row r="152" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A152" s="6">
-        <v>45078</v>
-      </c>
-      <c r="B152" s="14">
-        <v>5</v>
-      </c>
-      <c r="C152" s="11">
-        <v>0.25</v>
-      </c>
-      <c r="D152" s="7" t="s">
-        <v>11</v>
-      </c>
+      <c r="A152" s="6"/>
+      <c r="B152" s="14"/>
+      <c r="C152" s="11"/>
+      <c r="D152" s="7"/>
       <c r="E152" s="8" t="s">
-        <v>143</v>
+        <v>30</v>
       </c>
       <c r="F152" s="8"/>
     </row>
     <row r="153" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A153" s="6">
-        <v>45078</v>
-      </c>
-      <c r="B153" s="14">
-        <v>5</v>
-      </c>
-      <c r="C153" s="11">
-        <v>0.75</v>
-      </c>
-      <c r="D153" s="7" t="s">
-        <v>11</v>
-      </c>
+      <c r="A153" s="6"/>
+      <c r="B153" s="14"/>
+      <c r="C153" s="11"/>
+      <c r="D153" s="7"/>
       <c r="E153" s="8" t="s">
-        <v>144</v>
+        <v>31</v>
       </c>
       <c r="F153" s="8"/>
     </row>
     <row r="154" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A154" s="6">
-        <v>45078</v>
-      </c>
-      <c r="B154" s="14">
-        <v>5</v>
-      </c>
-      <c r="C154" s="11">
-        <v>0.5</v>
-      </c>
-      <c r="D154" s="7" t="s">
-        <v>6</v>
-      </c>
+      <c r="A154" s="6"/>
+      <c r="B154" s="14"/>
+      <c r="C154" s="11"/>
+      <c r="D154" s="7"/>
       <c r="E154" s="8" t="s">
-        <v>128</v>
+        <v>18</v>
       </c>
       <c r="F154" s="8"/>
     </row>
     <row r="155" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A155" s="6">
-        <v>45079</v>
-      </c>
-      <c r="B155" s="14">
-        <v>5</v>
-      </c>
-      <c r="C155" s="11">
-        <v>1</v>
-      </c>
-      <c r="D155" s="7" t="s">
-        <v>9</v>
-      </c>
+      <c r="A155" s="6"/>
+      <c r="B155" s="14"/>
+      <c r="C155" s="11"/>
+      <c r="D155" s="7"/>
       <c r="E155" s="8" t="s">
-        <v>145</v>
+        <v>32</v>
       </c>
       <c r="F155" s="8"/>
     </row>
     <row r="156" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A156" s="6">
-        <v>45079</v>
-      </c>
-      <c r="B156" s="14">
-        <v>5</v>
-      </c>
-      <c r="C156" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D156" s="7" t="s">
-        <v>11</v>
-      </c>
+      <c r="A156" s="6"/>
+      <c r="B156" s="14"/>
+      <c r="C156" s="11"/>
+      <c r="D156" s="7"/>
       <c r="E156" s="8" t="s">
         <v>15</v>
       </c>
       <c r="F156" s="8"/>
     </row>
     <row r="157" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A157" s="6">
-        <v>45079</v>
-      </c>
-      <c r="B157" s="14">
-        <v>5</v>
-      </c>
-      <c r="C157" s="11">
-        <v>1</v>
-      </c>
-      <c r="D157" s="7" t="s">
-        <v>11</v>
-      </c>
+      <c r="A157" s="6"/>
+      <c r="B157" s="14"/>
+      <c r="C157" s="11"/>
+      <c r="D157" s="7"/>
       <c r="E157" s="8" t="s">
-        <v>146</v>
+        <v>33</v>
       </c>
       <c r="F157" s="8"/>
     </row>
     <row r="158" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A158" s="6">
-        <v>45079</v>
-      </c>
-      <c r="B158" s="14">
-        <v>5</v>
-      </c>
-      <c r="C158" s="11">
-        <v>0.75</v>
-      </c>
-      <c r="D158" s="7" t="s">
-        <v>6</v>
-      </c>
+      <c r="A158" s="6"/>
+      <c r="B158" s="14"/>
+      <c r="C158" s="11"/>
+      <c r="D158" s="7"/>
       <c r="E158" s="8" t="s">
-        <v>147</v>
+        <v>34</v>
       </c>
       <c r="F158" s="8"/>
     </row>
     <row r="159" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A159" s="6">
-        <v>45079</v>
-      </c>
-      <c r="B159" s="14">
-        <v>5</v>
-      </c>
-      <c r="C159" s="11">
-        <v>1.25</v>
-      </c>
-      <c r="D159" s="7" t="s">
-        <v>6</v>
-      </c>
+      <c r="A159" s="6"/>
+      <c r="B159" s="14"/>
+      <c r="C159" s="11"/>
+      <c r="D159" s="7"/>
       <c r="E159" s="8" t="s">
-        <v>128</v>
+        <v>18</v>
       </c>
       <c r="F159" s="8"/>
     </row>
     <row r="160" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A160" s="6">
-        <v>45079</v>
-      </c>
-      <c r="B160" s="14">
-        <v>5</v>
-      </c>
-      <c r="C160" s="11">
-        <v>2.5</v>
-      </c>
-      <c r="D160" s="7" t="s">
-        <v>11</v>
-      </c>
+      <c r="A160" s="6"/>
+      <c r="B160" s="14"/>
+      <c r="C160" s="11"/>
+      <c r="D160" s="7"/>
       <c r="E160" s="8" t="s">
-        <v>148</v>
+        <v>35</v>
       </c>
       <c r="F160" s="8"/>
     </row>
@@ -7721,12 +6244,13 @@
       <c r="F500" s="8"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7:B300 B1:B5" xr:uid="{E1FCDE41-ACF1-4A68-9483-C062BB428146}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B5 B7:B300" xr:uid="{E1FCDE41-ACF1-4A68-9483-C062BB428146}">
       <formula1>1</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C300 C1:C5" xr:uid="{48106778-5E48-49BE-9E53-EB975C533ABF}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C5 C7:C300" xr:uid="{48106778-5E48-49BE-9E53-EB975C533ABF}">
       <formula1>0.25</formula1>
       <formula2>10</formula2>
     </dataValidation>
@@ -7777,7 +6301,7 @@
       </c>
       <c r="B2" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>11.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -7786,7 +6310,7 @@
       </c>
       <c r="B3" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>2.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -7795,7 +6319,7 @@
       </c>
       <c r="B4" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>125.75</v>
+        <v>12.75</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -7804,7 +6328,7 @@
       </c>
       <c r="B5" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>3.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -7813,7 +6337,7 @@
       </c>
       <c r="B6" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -7822,7 +6346,7 @@
       </c>
       <c r="B7" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>28.75</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -7840,7 +6364,7 @@
       </c>
       <c r="B9" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>0</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>